<commit_message>
4 DECEMBER 2025 CLOSING
</commit_message>
<xml_diff>
--- a/Daily Activities.xlsx
+++ b/Daily Activities.xlsx
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1421" uniqueCount="491">
   <si>
     <t>DATE</t>
   </si>
@@ -949,6 +949,30 @@
   </si>
   <si>
     <t>Picking up urgent Kitchen order 5 canned peeled tomatoes from Bu Bunga</t>
+  </si>
+  <si>
+    <t>Find rental places fr refrigerator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bar essential look for smaller cocktail </t>
+  </si>
+  <si>
+    <t>Purchase dimmer with bigger capacity than 200w led on local shop</t>
+  </si>
+  <si>
+    <t>Go to DIY look for 2 beautiful big glass and 1 Christmas tree lights</t>
+  </si>
+  <si>
+    <t>Check for price change on supplier and ask them when it's rising</t>
+  </si>
+  <si>
+    <t>Print 10 sticker on Balistars. Vinyl quality</t>
+  </si>
+  <si>
+    <t>Find glass cleaner robot on Tokopedia</t>
+  </si>
+  <si>
+    <t>Arrange to borrow 2 ice box from warung eka</t>
   </si>
   <si>
     <t>Date</t>
@@ -2476,7 +2500,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="152">
+  <cellXfs count="151">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -2927,11 +2951,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -4881,7 +4902,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K437"/>
+  <dimension ref="A1:K445"/>
   <sheetFormatPr defaultColWidth="9.16190476190476" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.8571428571429" style="114"/>
@@ -9517,7 +9538,7 @@
       </c>
     </row>
     <row r="412" spans="1:4">
-      <c r="A412" s="146">
+      <c r="A412" s="130">
         <v>45994</v>
       </c>
       <c r="B412" s="141" t="s">
@@ -9531,7 +9552,7 @@
       </c>
     </row>
     <row r="413" spans="1:4">
-      <c r="A413" s="147"/>
+      <c r="A413" s="123"/>
       <c r="B413" s="141" t="s">
         <v>144</v>
       </c>
@@ -9543,7 +9564,7 @@
       </c>
     </row>
     <row r="414" spans="1:4">
-      <c r="A414" s="147"/>
+      <c r="A414" s="123"/>
       <c r="B414" s="127" t="s">
         <v>107</v>
       </c>
@@ -9555,7 +9576,7 @@
       </c>
     </row>
     <row r="415" spans="1:4">
-      <c r="A415" s="147"/>
+      <c r="A415" s="123"/>
       <c r="B415" s="127" t="s">
         <v>172</v>
       </c>
@@ -9567,7 +9588,7 @@
       </c>
     </row>
     <row r="416" spans="1:4">
-      <c r="A416" s="147"/>
+      <c r="A416" s="123"/>
       <c r="B416" s="127" t="s">
         <v>238</v>
       </c>
@@ -9579,7 +9600,7 @@
       </c>
     </row>
     <row r="417" spans="1:4">
-      <c r="A417" s="147"/>
+      <c r="A417" s="123"/>
       <c r="B417" s="127" t="s">
         <v>259</v>
       </c>
@@ -9591,7 +9612,7 @@
       </c>
     </row>
     <row r="418" spans="1:4">
-      <c r="A418" s="147"/>
+      <c r="A418" s="123"/>
       <c r="B418" s="127" t="s">
         <v>271</v>
       </c>
@@ -9603,7 +9624,7 @@
       </c>
     </row>
     <row r="419" spans="1:4">
-      <c r="A419" s="147"/>
+      <c r="A419" s="123"/>
       <c r="B419" s="127" t="s">
         <v>272</v>
       </c>
@@ -9615,7 +9636,7 @@
       </c>
     </row>
     <row r="420" spans="1:4">
-      <c r="A420" s="147"/>
+      <c r="A420" s="123"/>
       <c r="B420" s="127" t="s">
         <v>279</v>
       </c>
@@ -9627,7 +9648,7 @@
       </c>
     </row>
     <row r="421" spans="1:4">
-      <c r="A421" s="147"/>
+      <c r="A421" s="123"/>
       <c r="B421" s="127" t="s">
         <v>283</v>
       </c>
@@ -9639,7 +9660,7 @@
       </c>
     </row>
     <row r="422" spans="1:4">
-      <c r="A422" s="147"/>
+      <c r="A422" s="123"/>
       <c r="B422" s="127" t="s">
         <v>284</v>
       </c>
@@ -9651,7 +9672,7 @@
       </c>
     </row>
     <row r="423" spans="1:4">
-      <c r="A423" s="147"/>
+      <c r="A423" s="123"/>
       <c r="B423" s="127" t="s">
         <v>287</v>
       </c>
@@ -9663,7 +9684,7 @@
       </c>
     </row>
     <row r="424" spans="1:4">
-      <c r="A424" s="147"/>
+      <c r="A424" s="123"/>
       <c r="B424" s="127" t="s">
         <v>288</v>
       </c>
@@ -9675,7 +9696,7 @@
       </c>
     </row>
     <row r="425" spans="1:4">
-      <c r="A425" s="147"/>
+      <c r="A425" s="123"/>
       <c r="B425" s="127" t="s">
         <v>294</v>
       </c>
@@ -9687,11 +9708,11 @@
       </c>
     </row>
     <row r="426" spans="1:4">
-      <c r="A426" s="148"/>
-      <c r="B426" s="149" t="s">
+      <c r="A426" s="129"/>
+      <c r="B426" s="127" t="s">
         <v>295</v>
       </c>
-      <c r="C426" s="150" t="s">
+      <c r="C426" s="128" t="s">
         <v>171</v>
       </c>
       <c r="D426" s="131" t="s">
@@ -9699,7 +9720,7 @@
       </c>
     </row>
     <row r="428" spans="1:4">
-      <c r="A428" s="151">
+      <c r="A428" s="146">
         <v>45994</v>
       </c>
       <c r="B428" s="141" t="s">
@@ -9713,7 +9734,7 @@
       </c>
     </row>
     <row r="429" spans="1:4">
-      <c r="A429" s="151"/>
+      <c r="A429" s="147"/>
       <c r="B429" s="141" t="s">
         <v>144</v>
       </c>
@@ -9725,7 +9746,7 @@
       </c>
     </row>
     <row r="430" spans="1:4">
-      <c r="A430" s="151"/>
+      <c r="A430" s="147"/>
       <c r="B430" s="127" t="s">
         <v>107</v>
       </c>
@@ -9737,7 +9758,7 @@
       </c>
     </row>
     <row r="431" spans="1:4">
-      <c r="A431" s="151"/>
+      <c r="A431" s="147"/>
       <c r="B431" s="127" t="s">
         <v>172</v>
       </c>
@@ -9749,7 +9770,7 @@
       </c>
     </row>
     <row r="432" spans="1:4">
-      <c r="A432" s="151"/>
+      <c r="A432" s="147"/>
       <c r="B432" s="127" t="s">
         <v>259</v>
       </c>
@@ -9761,7 +9782,7 @@
       </c>
     </row>
     <row r="433" spans="1:4">
-      <c r="A433" s="151"/>
+      <c r="A433" s="147"/>
       <c r="B433" s="127" t="s">
         <v>271</v>
       </c>
@@ -9773,7 +9794,7 @@
       </c>
     </row>
     <row r="434" spans="1:4">
-      <c r="A434" s="151"/>
+      <c r="A434" s="147"/>
       <c r="B434" s="127" t="s">
         <v>272</v>
       </c>
@@ -9785,7 +9806,7 @@
       </c>
     </row>
     <row r="435" spans="1:4">
-      <c r="A435" s="151"/>
+      <c r="A435" s="147"/>
       <c r="B435" s="127" t="s">
         <v>279</v>
       </c>
@@ -9797,7 +9818,7 @@
       </c>
     </row>
     <row r="436" spans="1:4">
-      <c r="A436" s="151"/>
+      <c r="A436" s="147"/>
       <c r="B436" s="127" t="s">
         <v>287</v>
       </c>
@@ -9809,7 +9830,7 @@
       </c>
     </row>
     <row r="437" spans="1:4">
-      <c r="A437" s="151"/>
+      <c r="A437" s="147"/>
       <c r="B437" s="127" t="s">
         <v>294</v>
       </c>
@@ -9817,6 +9838,102 @@
         <v>269</v>
       </c>
       <c r="D437" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="438" spans="1:4">
+      <c r="A438" s="147"/>
+      <c r="B438" s="127" t="s">
+        <v>296</v>
+      </c>
+      <c r="C438" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D438" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="439" spans="1:4">
+      <c r="A439" s="147"/>
+      <c r="B439" s="127" t="s">
+        <v>297</v>
+      </c>
+      <c r="C439" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D439" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="440" spans="1:4">
+      <c r="A440" s="147"/>
+      <c r="B440" s="127" t="s">
+        <v>298</v>
+      </c>
+      <c r="C440" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D440" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="441" spans="1:4">
+      <c r="A441" s="147"/>
+      <c r="B441" s="127" t="s">
+        <v>299</v>
+      </c>
+      <c r="C441" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D441" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="442" spans="1:4">
+      <c r="A442" s="147"/>
+      <c r="B442" s="127" t="s">
+        <v>300</v>
+      </c>
+      <c r="C442" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D442" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="443" spans="1:4">
+      <c r="A443" s="147"/>
+      <c r="B443" s="127" t="s">
+        <v>301</v>
+      </c>
+      <c r="C443" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D443" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="444" spans="1:4">
+      <c r="A444" s="147"/>
+      <c r="B444" s="127" t="s">
+        <v>302</v>
+      </c>
+      <c r="C444" s="137" t="s">
+        <v>269</v>
+      </c>
+      <c r="D444" s="131" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="445" spans="1:4">
+      <c r="A445" s="148"/>
+      <c r="B445" s="149" t="s">
+        <v>303</v>
+      </c>
+      <c r="C445" s="150" t="s">
+        <v>269</v>
+      </c>
+      <c r="D445" s="131" t="s">
         <v>47</v>
       </c>
     </row>
@@ -9853,7 +9970,7 @@
     <mergeCell ref="A384:A396"/>
     <mergeCell ref="A398:A410"/>
     <mergeCell ref="A412:A426"/>
-    <mergeCell ref="A428:A437"/>
+    <mergeCell ref="A428:A445"/>
     <mergeCell ref="D24:D25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9890,32 +10007,32 @@
   <sheetData>
     <row r="1" s="76" customFormat="1" spans="1:10">
       <c r="A1" s="84" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="B1" s="84" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="C1" s="84" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="D1" s="84" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="E1" s="84" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="F1" s="85" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="G1" s="84" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="H1" s="84" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="I1" s="108"/>
       <c r="J1" s="109" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -9923,10 +10040,10 @@
         <v>45954</v>
       </c>
       <c r="B2" s="87" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C2" s="88" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="D2" s="89">
         <v>16</v>
@@ -9953,10 +10070,10 @@
         <v>45956</v>
       </c>
       <c r="B3" s="93" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C3" s="94" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="D3" s="95">
         <v>5.7</v>
@@ -9972,16 +10089,16 @@
       <c r="G3" s="94"/>
       <c r="H3" s="97"/>
       <c r="J3" s="109" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="92"/>
       <c r="B4" s="93" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C4" s="94" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="D4" s="95">
         <v>3.5</v>
@@ -10000,10 +10117,10 @@
     <row r="5" s="77" customFormat="1" spans="1:10">
       <c r="A5" s="92"/>
       <c r="B5" s="93" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="C5" s="94" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="D5" s="95">
         <v>5.8</v>
@@ -10017,7 +10134,7 @@
       <c r="H5" s="97"/>
       <c r="I5" s="76"/>
       <c r="J5" s="109" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -10025,10 +10142,10 @@
         <v>45957</v>
       </c>
       <c r="B6" s="87" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="C6" s="88" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
       <c r="D6" s="89">
         <v>23</v>
@@ -10053,10 +10170,10 @@
         <v>45958</v>
       </c>
       <c r="B7" s="93" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C7" s="94" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="D7" s="95">
         <v>23</v>
@@ -10073,16 +10190,16 @@
       <c r="H7" s="97"/>
       <c r="I7" s="76"/>
       <c r="J7" s="109" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="92"/>
       <c r="B8" s="93" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="C8" s="94" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="D8" s="95">
         <v>5.3</v>
@@ -10104,10 +10221,10 @@
         <v>45959</v>
       </c>
       <c r="B9" s="87" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
       <c r="C9" s="88" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="D9" s="89">
         <v>30</v>
@@ -10124,7 +10241,7 @@
       <c r="H9" s="97"/>
       <c r="I9" s="76"/>
       <c r="J9" s="109" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -10132,10 +10249,10 @@
         <v>45960</v>
       </c>
       <c r="B10" s="93" t="s">
-        <v>325</v>
+        <v>333</v>
       </c>
       <c r="C10" s="94" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="D10" s="95">
         <v>30</v>
@@ -10157,10 +10274,10 @@
     <row r="11" spans="1:10">
       <c r="A11" s="92"/>
       <c r="B11" s="93" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C11" s="94" t="s">
-        <v>328</v>
+        <v>336</v>
       </c>
       <c r="D11" s="95">
         <v>11</v>
@@ -10174,16 +10291,16 @@
       <c r="H11" s="97"/>
       <c r="I11" s="76"/>
       <c r="J11" s="112" t="s">
-        <v>329</v>
+        <v>337</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="92"/>
       <c r="B12" s="93" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="C12" s="94" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="D12" s="95">
         <v>12</v>
@@ -10203,10 +10320,10 @@
     <row r="13" spans="1:10">
       <c r="A13" s="92"/>
       <c r="B13" s="93" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="C13" s="94" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="D13" s="95">
         <v>11</v>
@@ -10220,16 +10337,16 @@
       <c r="H13" s="97"/>
       <c r="I13" s="76"/>
       <c r="J13" s="112" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="92"/>
       <c r="B14" s="93" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="C14" s="94" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="D14" s="95">
         <v>12</v>
@@ -10249,10 +10366,10 @@
     <row r="15" spans="1:10">
       <c r="A15" s="92"/>
       <c r="B15" s="93" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="C15" s="94" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="D15" s="95">
         <v>13.2</v>
@@ -10266,7 +10383,7 @@
       <c r="H15" s="97"/>
       <c r="I15" s="76"/>
       <c r="J15" s="112" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -10274,10 +10391,10 @@
         <v>45961</v>
       </c>
       <c r="B16" s="87" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C16" s="88" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="D16" s="89">
         <v>11.4</v>
@@ -10300,10 +10417,10 @@
     <row r="17" spans="1:10">
       <c r="A17" s="86"/>
       <c r="B17" s="87" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="C17" s="88" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="D17" s="89">
         <v>12.6</v>
@@ -10317,7 +10434,7 @@
       <c r="H17" s="97"/>
       <c r="I17" s="76"/>
       <c r="J17" s="113" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -10325,10 +10442,10 @@
         <v>45964</v>
       </c>
       <c r="B18" s="93" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="C18" s="94" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="D18" s="95">
         <v>24</v>
@@ -10351,10 +10468,10 @@
     <row r="19" spans="1:9">
       <c r="A19" s="92"/>
       <c r="B19" s="93" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="C19" s="94" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="D19" s="95">
         <v>13.4</v>
@@ -10373,10 +10490,10 @@
         <v>45966</v>
       </c>
       <c r="B20" s="99" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="C20" s="100" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="D20" s="101">
         <v>8.2</v>
@@ -10395,10 +10512,10 @@
     <row r="21" spans="1:9">
       <c r="A21" s="98"/>
       <c r="B21" s="99" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
       <c r="C21" s="100" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="D21" s="101">
         <v>27</v>
@@ -10415,10 +10532,10 @@
     <row r="22" spans="1:8">
       <c r="A22" s="98"/>
       <c r="B22" s="99" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C22" s="100" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="D22" s="101">
         <v>22</v>
@@ -10436,10 +10553,10 @@
         <v>45967</v>
       </c>
       <c r="B23" s="94" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="C23" s="94" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="D23" s="95">
         <v>24</v>
@@ -10458,10 +10575,10 @@
     <row r="24" spans="1:8">
       <c r="A24" s="92"/>
       <c r="B24" s="93" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="C24" s="94" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="D24" s="95">
         <v>12</v>
@@ -10479,10 +10596,10 @@
         <v>45969</v>
       </c>
       <c r="B25" s="99" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C25" s="100" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="D25" s="101">
         <v>12.4</v>
@@ -10503,10 +10620,10 @@
         <v>45971</v>
       </c>
       <c r="B26" s="93" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C26" s="94" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="D26" s="95">
         <v>15.8</v>
@@ -10527,10 +10644,10 @@
         <v>45972</v>
       </c>
       <c r="B27" s="99" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C27" s="100" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="D27" s="101">
         <v>13</v>
@@ -10551,10 +10668,10 @@
         <v>45974</v>
       </c>
       <c r="B28" s="93" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C28" s="94" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="D28" s="95">
         <v>15</v>
@@ -10573,10 +10690,10 @@
     <row r="29" spans="1:8">
       <c r="A29" s="92"/>
       <c r="B29" s="93" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C29" s="94" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="D29" s="95">
         <v>20</v>
@@ -10594,10 +10711,10 @@
         <v>45979</v>
       </c>
       <c r="B30" s="99" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C30" s="100" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="D30" s="101">
         <v>12</v>
@@ -10618,10 +10735,10 @@
         <v>45980</v>
       </c>
       <c r="B31" s="93" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="C31" s="94" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="D31" s="95">
         <v>10.9</v>
@@ -10640,10 +10757,10 @@
     <row r="32" spans="1:8">
       <c r="A32" s="92"/>
       <c r="B32" s="93" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="C32" s="94" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="D32" s="95">
         <v>18</v>
@@ -10661,10 +10778,10 @@
         <v>45982</v>
       </c>
       <c r="B33" s="99" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="C33" s="100" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="D33" s="101">
         <v>3.6</v>
@@ -10683,10 +10800,10 @@
     <row r="34" spans="1:8">
       <c r="A34" s="98"/>
       <c r="B34" s="99" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="C34" s="100" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="D34" s="101">
         <v>16</v>
@@ -10702,10 +10819,10 @@
     <row r="35" spans="1:8">
       <c r="A35" s="98"/>
       <c r="B35" s="99" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="C35" s="100" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="D35" s="101">
         <v>13.4</v>
@@ -10721,10 +10838,10 @@
     <row r="36" spans="1:8">
       <c r="A36" s="98"/>
       <c r="B36" s="99" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C36" s="100" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="D36" s="101">
         <v>12</v>
@@ -10740,10 +10857,10 @@
     <row r="37" spans="1:8">
       <c r="A37" s="98"/>
       <c r="B37" s="99" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="C37" s="100" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="D37" s="101">
         <v>16.4</v>
@@ -10761,10 +10878,10 @@
         <v>45983</v>
       </c>
       <c r="B38" s="93" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="C38" s="94" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="D38" s="95">
         <v>14</v>
@@ -10785,10 +10902,10 @@
         <v>45987</v>
       </c>
       <c r="B39" s="99" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="C39" s="100" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="D39" s="101">
         <v>16</v>
@@ -10807,10 +10924,10 @@
     <row r="40" spans="1:8">
       <c r="A40" s="98"/>
       <c r="B40" s="99" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="C40" s="100" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="D40" s="101">
         <v>12.4</v>
@@ -10828,10 +10945,10 @@
         <v>45988</v>
       </c>
       <c r="B41" s="93" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="C41" s="94" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="D41" s="95">
         <v>22</v>
@@ -10850,10 +10967,10 @@
     <row r="42" spans="1:8">
       <c r="A42" s="92"/>
       <c r="B42" s="93" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="C42" s="94" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="D42" s="95">
         <v>13.2</v>
@@ -10871,10 +10988,10 @@
         <v>45990</v>
       </c>
       <c r="B43" s="99" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="C43" s="100" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="D43" s="101">
         <v>15.2</v>
@@ -10895,10 +11012,10 @@
         <v>45992</v>
       </c>
       <c r="B44" s="93" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="C44" s="94" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="D44" s="95">
         <v>2.8</v>
@@ -10917,10 +11034,10 @@
     <row r="45" spans="1:8">
       <c r="A45" s="92"/>
       <c r="B45" s="93" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="C45" s="94" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="D45" s="95">
         <v>16</v>
@@ -10990,31 +11107,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="59" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="C1" s="60" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="D1" s="60" t="s">
-        <v>397</v>
+        <v>405</v>
       </c>
       <c r="E1" s="59" t="s">
-        <v>398</v>
+        <v>406</v>
       </c>
       <c r="F1" s="59" t="s">
-        <v>399</v>
+        <v>407</v>
       </c>
       <c r="G1" s="61" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="H1" s="61" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="I1" s="61" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="J1" s="59" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" ht="129" customHeight="1" spans="1:10">
@@ -11022,16 +11139,16 @@
         <v>45967</v>
       </c>
       <c r="B2" s="63" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="C2" s="64" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="D2" s="65">
         <v>3</v>
       </c>
       <c r="E2" s="66" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="F2" s="66" t="str">
         <f>_xlfn.DISPIMG("ID_A435215B813C404CA26F65668F85307D",1)</f>
@@ -11049,7 +11166,7 @@
         <v>846000</v>
       </c>
       <c r="J2" s="66" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
     </row>
     <row r="3" ht="43" customHeight="1" spans="1:10">
@@ -11231,25 +11348,25 @@
   <sheetData>
     <row r="1" ht="39.75" customHeight="1" spans="1:56">
       <c r="A1" s="3" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="H1" s="7"/>
       <c r="I1" s="7"/>
@@ -11306,7 +11423,7 @@
         <v>45973</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="C2" s="10">
         <v>1000000</v>
@@ -11317,7 +11434,7 @@
         <v>1000000</v>
       </c>
       <c r="F2" s="13" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="15"/>
@@ -11375,7 +11492,7 @@
         <v>45973</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="11">
@@ -11386,7 +11503,7 @@
         <v>998800</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="G3" s="16"/>
       <c r="H3" s="15"/>
@@ -11444,7 +11561,7 @@
         <v>45974</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="C4" s="10"/>
       <c r="D4" s="11">
@@ -11455,7 +11572,7 @@
         <v>948800</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="15"/>
@@ -11513,7 +11630,7 @@
         <v>45974</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="C5" s="10"/>
       <c r="D5" s="11">
@@ -11524,7 +11641,7 @@
         <v>693800</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>422</v>
+        <v>430</v>
       </c>
       <c r="G5" s="19"/>
       <c r="H5" s="15"/>
@@ -11582,7 +11699,7 @@
         <v>45974</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>423</v>
+        <v>431</v>
       </c>
       <c r="C6" s="10"/>
       <c r="D6" s="11">
@@ -11593,7 +11710,7 @@
         <v>682800</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>424</v>
+        <v>432</v>
       </c>
       <c r="G6" s="17"/>
       <c r="H6" s="15"/>
@@ -11651,7 +11768,7 @@
         <v>45974</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>425</v>
+        <v>433</v>
       </c>
       <c r="C7" s="10"/>
       <c r="D7" s="11">
@@ -11662,7 +11779,7 @@
         <v>569800</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>426</v>
+        <v>434</v>
       </c>
       <c r="G7" s="19"/>
       <c r="H7" s="15"/>
@@ -11720,7 +11837,7 @@
         <v>45975</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>427</v>
+        <v>435</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="11">
@@ -11731,7 +11848,7 @@
         <v>551800</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="G8" s="20"/>
       <c r="H8" s="15"/>
@@ -11789,7 +11906,7 @@
         <v>45975</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="11">
@@ -11800,7 +11917,7 @@
         <v>515300</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="G9" s="19"/>
       <c r="H9" s="15"/>
@@ -11858,7 +11975,7 @@
         <v>45978</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="C10" s="10"/>
       <c r="D10" s="11">
@@ -11869,7 +11986,7 @@
         <v>329800</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="G10" s="20"/>
       <c r="H10" s="15"/>
@@ -11927,7 +12044,7 @@
         <v>45979</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>431</v>
+        <v>439</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="11">
@@ -11938,7 +12055,7 @@
         <v>302300</v>
       </c>
       <c r="F11" s="13" t="s">
-        <v>433</v>
+        <v>441</v>
       </c>
       <c r="G11" s="19"/>
       <c r="H11" s="15"/>
@@ -11996,7 +12113,7 @@
         <v>45979</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="C12" s="10"/>
       <c r="D12" s="11">
@@ -12007,7 +12124,7 @@
         <v>218300</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="G12" s="20"/>
       <c r="H12" s="15"/>
@@ -12065,7 +12182,7 @@
         <v>45980</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>436</v>
+        <v>444</v>
       </c>
       <c r="C13" s="10"/>
       <c r="D13" s="11">
@@ -12076,7 +12193,7 @@
         <v>165400</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>437</v>
+        <v>445</v>
       </c>
       <c r="G13" s="19"/>
       <c r="H13" s="15"/>
@@ -12134,7 +12251,7 @@
         <v>45980</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C14" s="10"/>
       <c r="D14" s="11">
@@ -12145,14 +12262,14 @@
         <v>115400</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>439</v>
+        <v>447</v>
       </c>
       <c r="G14" s="17"/>
       <c r="H14" s="15" t="s">
-        <v>440</v>
+        <v>448</v>
       </c>
       <c r="I14" s="15" t="s">
-        <v>441</v>
+        <v>449</v>
       </c>
       <c r="J14" s="15"/>
       <c r="K14" s="15"/>
@@ -12207,7 +12324,7 @@
         <v>45982</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>442</v>
+        <v>450</v>
       </c>
       <c r="C15" s="21"/>
       <c r="D15" s="11">
@@ -12218,7 +12335,7 @@
         <v>89400</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>443</v>
+        <v>451</v>
       </c>
       <c r="G15" s="22"/>
       <c r="H15" s="15"/>
@@ -12276,7 +12393,7 @@
         <v>45982</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>444</v>
+        <v>452</v>
       </c>
       <c r="C16" s="25"/>
       <c r="D16" s="26">
@@ -12287,7 +12404,7 @@
         <v>28700</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>445</v>
+        <v>453</v>
       </c>
       <c r="G16" s="20"/>
       <c r="H16" s="15"/>
@@ -12347,7 +12464,7 @@
       <c r="D17" s="29"/>
       <c r="E17" s="30"/>
       <c r="F17" s="13" t="s">
-        <v>446</v>
+        <v>454</v>
       </c>
       <c r="G17" s="31"/>
       <c r="H17" s="15"/>
@@ -12407,7 +12524,7 @@
       <c r="D18" s="34"/>
       <c r="E18" s="35"/>
       <c r="F18" s="13" t="s">
-        <v>447</v>
+        <v>455</v>
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="15"/>
@@ -12465,7 +12582,7 @@
         <v>45986</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="C19" s="10">
         <v>1000000</v>
@@ -12476,7 +12593,7 @@
         <v>1028700</v>
       </c>
       <c r="F19" s="13" t="s">
-        <v>448</v>
+        <v>456</v>
       </c>
       <c r="G19" s="36"/>
       <c r="H19" s="15"/>
@@ -12534,7 +12651,7 @@
         <v>45986</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C20" s="10"/>
       <c r="D20" s="11">
@@ -12545,7 +12662,7 @@
         <v>1027500</v>
       </c>
       <c r="F20" s="13" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="G20" s="37"/>
       <c r="H20" s="15"/>
@@ -12603,7 +12720,7 @@
         <v>45987</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="11">
@@ -12614,7 +12731,7 @@
         <v>1022500</v>
       </c>
       <c r="F21" s="13" t="s">
-        <v>449</v>
+        <v>457</v>
       </c>
       <c r="G21" s="31"/>
       <c r="H21" s="15"/>
@@ -12672,7 +12789,7 @@
         <v>45987</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="11">
@@ -12683,7 +12800,7 @@
         <v>1009750</v>
       </c>
       <c r="F22" s="13" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="G22" s="20"/>
       <c r="H22" s="15"/>
@@ -12741,7 +12858,7 @@
         <v>45987</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>452</v>
+        <v>460</v>
       </c>
       <c r="C23" s="10"/>
       <c r="D23" s="11">
@@ -12752,7 +12869,7 @@
         <v>707250</v>
       </c>
       <c r="F23" s="13" t="s">
-        <v>453</v>
+        <v>461</v>
       </c>
       <c r="G23" s="31"/>
       <c r="H23" s="15"/>
@@ -12810,7 +12927,7 @@
         <v>45987</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>454</v>
+        <v>462</v>
       </c>
       <c r="C24" s="10"/>
       <c r="D24" s="11">
@@ -12821,7 +12938,7 @@
         <v>618250</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>455</v>
+        <v>463</v>
       </c>
       <c r="G24" s="20"/>
       <c r="H24" s="7"/>
@@ -12879,7 +12996,7 @@
         <v>45988</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>456</v>
+        <v>464</v>
       </c>
       <c r="C25" s="10"/>
       <c r="D25" s="10">
@@ -12890,7 +13007,7 @@
         <v>508913</v>
       </c>
       <c r="F25" s="13" t="s">
-        <v>457</v>
+        <v>465</v>
       </c>
       <c r="G25" s="38"/>
       <c r="H25" s="15"/>
@@ -12948,7 +13065,7 @@
         <v>45988</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>458</v>
+        <v>466</v>
       </c>
       <c r="C26" s="10"/>
       <c r="D26" s="10">
@@ -12959,7 +13076,7 @@
         <v>473913</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>459</v>
+        <v>467</v>
       </c>
       <c r="G26" s="40"/>
       <c r="H26" s="15"/>
@@ -13017,7 +13134,7 @@
         <v>45988</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>460</v>
+        <v>468</v>
       </c>
       <c r="C27" s="10"/>
       <c r="D27" s="10">
@@ -13028,7 +13145,7 @@
         <v>333913</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>461</v>
+        <v>469</v>
       </c>
       <c r="G27" s="38"/>
       <c r="H27" s="15"/>
@@ -13086,7 +13203,7 @@
         <v>45988</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>462</v>
+        <v>470</v>
       </c>
       <c r="C28" s="10"/>
       <c r="D28" s="10">
@@ -13097,7 +13214,7 @@
         <v>289913</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>463</v>
+        <v>471</v>
       </c>
       <c r="G28" s="40"/>
       <c r="H28" s="15"/>
@@ -13155,7 +13272,7 @@
         <v>45988</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>464</v>
+        <v>472</v>
       </c>
       <c r="C29" s="10"/>
       <c r="D29" s="10">
@@ -13166,7 +13283,7 @@
         <v>265913</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>465</v>
+        <v>473</v>
       </c>
       <c r="G29" s="38"/>
       <c r="H29" s="15"/>
@@ -13224,7 +13341,7 @@
         <v>45989</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>466</v>
+        <v>474</v>
       </c>
       <c r="C30" s="10">
         <v>1000000</v>
@@ -13235,7 +13352,7 @@
         <v>1265913</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="G30" s="40"/>
       <c r="H30" s="15"/>
@@ -13293,7 +13410,7 @@
         <v>45989</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="C31" s="10"/>
       <c r="D31" s="10">
@@ -13304,7 +13421,7 @@
         <v>1264913</v>
       </c>
       <c r="F31" s="13" t="s">
-        <v>467</v>
+        <v>475</v>
       </c>
       <c r="G31" s="40"/>
       <c r="H31" s="15"/>
@@ -13362,7 +13479,7 @@
         <v>45989</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>468</v>
+        <v>476</v>
       </c>
       <c r="C32" s="10"/>
       <c r="D32" s="10">
@@ -13373,7 +13490,7 @@
         <v>1109666</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>469</v>
+        <v>477</v>
       </c>
       <c r="G32" s="40"/>
       <c r="H32" s="15"/>
@@ -13431,7 +13548,7 @@
         <v>28</v>
       </c>
       <c r="B33" s="41" t="s">
-        <v>470</v>
+        <v>478</v>
       </c>
       <c r="C33" s="42">
         <v>810</v>
@@ -13442,7 +13559,7 @@
         <v>1110476</v>
       </c>
       <c r="F33" s="43" t="s">
-        <v>471</v>
+        <v>479</v>
       </c>
       <c r="G33" s="44"/>
       <c r="H33" s="15"/>
@@ -13500,7 +13617,7 @@
         <v>45990</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>472</v>
+        <v>480</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="11">
@@ -13511,7 +13628,7 @@
         <v>825476</v>
       </c>
       <c r="F34" s="45" t="s">
-        <v>473</v>
+        <v>481</v>
       </c>
       <c r="G34" s="40"/>
       <c r="H34" s="15"/>
@@ -13569,7 +13686,7 @@
         <v>45990</v>
       </c>
       <c r="B35" s="46" t="s">
-        <v>429</v>
+        <v>437</v>
       </c>
       <c r="C35" s="47"/>
       <c r="D35" s="47">
@@ -13580,7 +13697,7 @@
         <v>811476</v>
       </c>
       <c r="F35" s="48" t="s">
-        <v>474</v>
+        <v>482</v>
       </c>
       <c r="G35" s="49"/>
       <c r="H35" s="15"/>
@@ -13638,7 +13755,7 @@
         <v>45991</v>
       </c>
       <c r="B36" s="46" t="s">
-        <v>475</v>
+        <v>483</v>
       </c>
       <c r="C36" s="47"/>
       <c r="D36" s="47">
@@ -13649,7 +13766,7 @@
         <v>753976</v>
       </c>
       <c r="F36" s="48" t="s">
-        <v>476</v>
+        <v>484</v>
       </c>
       <c r="G36" s="49"/>
       <c r="H36" s="50"/>
@@ -13707,7 +13824,7 @@
         <v>45992</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>477</v>
+        <v>485</v>
       </c>
       <c r="C37" s="10"/>
       <c r="D37" s="11">
@@ -13718,7 +13835,7 @@
         <v>659976</v>
       </c>
       <c r="F37" s="45" t="s">
-        <v>478</v>
+        <v>486</v>
       </c>
       <c r="G37" s="40"/>
       <c r="H37" s="15"/>
@@ -13776,7 +13893,7 @@
         <v>45992</v>
       </c>
       <c r="B38" s="18" t="s">
-        <v>479</v>
+        <v>487</v>
       </c>
       <c r="C38" s="10"/>
       <c r="D38" s="11">
@@ -13787,7 +13904,7 @@
         <v>609976</v>
       </c>
       <c r="F38" s="45" t="s">
-        <v>480</v>
+        <v>488</v>
       </c>
       <c r="G38" s="38"/>
       <c r="H38" s="15"/>
@@ -13845,7 +13962,7 @@
         <v>45992</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>438</v>
+        <v>446</v>
       </c>
       <c r="C39" s="10"/>
       <c r="D39" s="11">
@@ -13856,7 +13973,7 @@
         <v>509976</v>
       </c>
       <c r="F39" s="45" t="s">
-        <v>481</v>
+        <v>489</v>
       </c>
       <c r="G39" s="40"/>
       <c r="H39" s="15"/>
@@ -13914,7 +14031,7 @@
         <v>45993</v>
       </c>
       <c r="B40" s="46" t="s">
-        <v>434</v>
+        <v>442</v>
       </c>
       <c r="C40" s="47"/>
       <c r="D40" s="47">
@@ -13925,7 +14042,7 @@
         <v>425976</v>
       </c>
       <c r="F40" s="48" t="s">
-        <v>435</v>
+        <v>443</v>
       </c>
       <c r="G40" s="49"/>
       <c r="H40" s="15"/>
@@ -16295,7 +16412,7 @@
       <c r="BB78" s="7"/>
       <c r="BC78" s="7"/>
       <c r="BD78" s="7" t="s">
-        <v>482</v>
+        <v>490</v>
       </c>
     </row>
     <row r="79" ht="39.75" customHeight="1" spans="1:56">

</xml_diff>

<commit_message>
Update 17th feb 2026 19:43
</commit_message>
<xml_diff>
--- a/Daily Activities.xlsx
+++ b/Daily Activities.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="15980" windowHeight="17020"/>
+    <workbookView windowWidth="11260" windowHeight="17020"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Acitivies &amp; Checklists" sheetId="26" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4191" uniqueCount="635">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4539" uniqueCount="654">
   <si>
     <t>DATE</t>
   </si>
@@ -1503,6 +1503,63 @@
   </si>
   <si>
     <t>Print flyers for ululani rooms</t>
+  </si>
+  <si>
+    <t>Done dimmer has arrived</t>
+  </si>
+  <si>
+    <t>Purchase water filter for ADVANCE drinking machine</t>
+  </si>
+  <si>
+    <t>on progress (already purchase)</t>
+  </si>
+  <si>
+    <t>Canvas and paint for art</t>
+  </si>
+  <si>
+    <t>Print floor sticker</t>
+  </si>
+  <si>
+    <t>Follow up for the service of water purifier</t>
+  </si>
+  <si>
+    <t>Purchase blue paint for bar ceilling</t>
+  </si>
+  <si>
+    <t>Peeler Victorinox 2 pcs on tokopedia</t>
+  </si>
+  <si>
+    <t>Purchase blue paint for bar ceilling Nippon 2020 matte</t>
+  </si>
+  <si>
+    <t>Peeler Victorinox &amp; mixer head 2 pcs on tokopedia</t>
+  </si>
+  <si>
+    <t>Posted on Lemesy</t>
+  </si>
+  <si>
+    <t>Print credit agreement for apperol supplier</t>
+  </si>
+  <si>
+    <t>Purchase bar lamp</t>
+  </si>
+  <si>
+    <t>Pick up Salami 4 kg from kemfood</t>
+  </si>
+  <si>
+    <t>On progress. Need to collect data to input and also owner sign</t>
+  </si>
+  <si>
+    <t>On progress (waiting for petty cash)</t>
+  </si>
+  <si>
+    <t>Purchase fruit knife for bar</t>
+  </si>
+  <si>
+    <t>Tortilla matang 6 bungkus</t>
+  </si>
+  <si>
+    <t>Purchase fox glue 2 pack</t>
   </si>
   <si>
     <t>Date</t>
@@ -2720,7 +2777,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="118">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3054,6 +3111,27 @@
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3364,7 +3442,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14245590" y="232724960"/>
+          <a:off x="10856595" y="232724960"/>
           <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3405,7 +3483,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14245590" y="236230160"/>
+          <a:off x="10856595" y="236230160"/>
           <a:ext cx="0" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -3724,12 +3802,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K1443"/>
+  <dimension ref="A1:K1567"/>
   <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12.859375" style="72"/>
-    <col min="2" max="2" width="67.9765625" customWidth="1"/>
-    <col min="3" max="3" width="94.4296875" style="73" customWidth="1"/>
+    <col min="2" max="2" width="60.8125" customWidth="1"/>
+    <col min="3" max="3" width="59.8984375" style="73" customWidth="1"/>
     <col min="4" max="4" width="9.1640625" style="74"/>
     <col min="6" max="6" width="12.828125"/>
     <col min="7" max="7" width="53.828125" customWidth="1"/>
@@ -20136,7 +20214,7 @@
         <v>488</v>
       </c>
       <c r="C1441" s="93" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D1441" s="1" t="s">
         <v>47</v>
@@ -20148,7 +20226,7 @@
         <v>489</v>
       </c>
       <c r="C1442" s="93" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="D1442" s="1" t="s">
         <v>47</v>
@@ -20166,8 +20244,1416 @@
         <v>47</v>
       </c>
     </row>
+    <row r="1445" spans="1:4">
+      <c r="A1445" s="86">
+        <v>46060</v>
+      </c>
+      <c r="B1445" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1445" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1445" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1446" spans="1:4">
+      <c r="A1446" s="80"/>
+      <c r="B1446" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1446" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1446" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1447" spans="1:4">
+      <c r="A1447" s="80"/>
+      <c r="B1447" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1447" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1447" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1448" spans="1:4">
+      <c r="A1448" s="80"/>
+      <c r="B1448" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1448" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1448" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1449" spans="1:4">
+      <c r="A1449" s="80"/>
+      <c r="B1449" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1449" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1449" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1450" spans="1:4">
+      <c r="A1450" s="80"/>
+      <c r="B1450" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1450" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1450" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1451" spans="1:4">
+      <c r="A1451" s="80"/>
+      <c r="B1451" s="2" t="s">
+        <v>482</v>
+      </c>
+      <c r="C1451" s="84" t="s">
+        <v>491</v>
+      </c>
+      <c r="D1451" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1452" spans="1:4">
+      <c r="A1452" s="80"/>
+      <c r="B1452" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C1452" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1452" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1453" spans="1:4">
+      <c r="A1453" s="80"/>
+      <c r="B1453" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1453" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1453" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1454" spans="1:4">
+      <c r="A1454" s="80"/>
+      <c r="B1454" s="2" t="s">
+        <v>486</v>
+      </c>
+      <c r="C1454" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1454" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1455" spans="1:4">
+      <c r="A1455" s="80"/>
+      <c r="B1455" s="2" t="s">
+        <v>487</v>
+      </c>
+      <c r="C1455" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1455" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1456" spans="1:4">
+      <c r="A1456" s="80"/>
+      <c r="B1456" s="2" t="s">
+        <v>488</v>
+      </c>
+      <c r="C1456" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1456" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1457" spans="1:4">
+      <c r="A1457" s="80"/>
+      <c r="B1457" s="2" t="s">
+        <v>489</v>
+      </c>
+      <c r="C1457" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1457" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1458" spans="1:4">
+      <c r="A1458" s="85"/>
+      <c r="B1458" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1458" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1458" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1460" spans="1:4">
+      <c r="A1460" s="86">
+        <v>46061</v>
+      </c>
+      <c r="B1460" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1460" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1460" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1461" spans="1:4">
+      <c r="A1461" s="80"/>
+      <c r="B1461" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1461" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1461" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1462" spans="1:4">
+      <c r="A1462" s="80"/>
+      <c r="B1462" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1462" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1462" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1463" spans="1:4">
+      <c r="A1463" s="80"/>
+      <c r="B1463" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1463" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1463" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1464" spans="1:4">
+      <c r="A1464" s="80"/>
+      <c r="B1464" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1464" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1464" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1465" spans="1:4">
+      <c r="A1465" s="80"/>
+      <c r="B1465" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1465" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1465" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1466" spans="1:4">
+      <c r="A1466" s="80"/>
+      <c r="B1466" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C1466" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1466" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1467" spans="1:4">
+      <c r="A1467" s="80"/>
+      <c r="B1467" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1467" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1467" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1468" spans="1:4">
+      <c r="A1468" s="85"/>
+      <c r="B1468" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1468" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1468" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1470" spans="1:4">
+      <c r="A1470" s="86">
+        <v>46063</v>
+      </c>
+      <c r="B1470" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1470" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1470" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1471" spans="1:4">
+      <c r="A1471" s="80"/>
+      <c r="B1471" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1471" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1471" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1472" spans="1:4">
+      <c r="A1472" s="80"/>
+      <c r="B1472" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1472" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1472" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1473" spans="1:4">
+      <c r="A1473" s="80"/>
+      <c r="B1473" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1473" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1473" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1474" spans="1:4">
+      <c r="A1474" s="80"/>
+      <c r="B1474" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1474" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1474" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1475" spans="1:4">
+      <c r="A1475" s="80"/>
+      <c r="B1475" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1475" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1475" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1476" spans="1:4">
+      <c r="A1476" s="80"/>
+      <c r="B1476" s="2" t="s">
+        <v>484</v>
+      </c>
+      <c r="C1476" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1476" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1477" spans="1:4">
+      <c r="A1477" s="80"/>
+      <c r="B1477" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1477" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1477" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1478" spans="1:4">
+      <c r="A1478" s="80"/>
+      <c r="B1478" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1478" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1478" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1479" spans="1:4">
+      <c r="A1479" s="80"/>
+      <c r="B1479" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="C1479" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1479" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1480" spans="1:4">
+      <c r="A1480" s="80"/>
+      <c r="B1480" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C1480" s="93" t="s">
+        <v>493</v>
+      </c>
+      <c r="D1480" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1481" spans="1:4">
+      <c r="A1481" s="80"/>
+      <c r="B1481" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1481" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1481" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1482" spans="1:4">
+      <c r="A1482" s="80"/>
+      <c r="B1482" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1482" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1482" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1483" spans="1:4">
+      <c r="A1483" s="85"/>
+      <c r="B1483" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1483" s="93" t="s">
+        <v>75</v>
+      </c>
+      <c r="D1483" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1485" spans="1:4">
+      <c r="A1485" s="86">
+        <v>46065</v>
+      </c>
+      <c r="B1485" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1485" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1485" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1486" spans="1:4">
+      <c r="A1486" s="80"/>
+      <c r="B1486" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1486" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1486" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1487" spans="1:4">
+      <c r="A1487" s="80"/>
+      <c r="B1487" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1487" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1487" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1488" spans="1:4">
+      <c r="A1488" s="80"/>
+      <c r="B1488" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1488" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1488" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1489" spans="1:4">
+      <c r="A1489" s="80"/>
+      <c r="B1489" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1489" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1489" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1490" spans="1:4">
+      <c r="A1490" s="80"/>
+      <c r="B1490" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1490" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1490" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1491" spans="1:4">
+      <c r="A1491" s="80"/>
+      <c r="B1491" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="C1491" s="84" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1491" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1492" spans="1:4">
+      <c r="A1492" s="80"/>
+      <c r="B1492" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1492" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1492" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1493" spans="1:4">
+      <c r="A1493" s="80"/>
+      <c r="B1493" s="2" t="s">
+        <v>492</v>
+      </c>
+      <c r="C1493" s="84" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1493" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1494" spans="1:4">
+      <c r="A1494" s="80"/>
+      <c r="B1494" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1494" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1494" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1495" spans="1:4">
+      <c r="A1495" s="80"/>
+      <c r="B1495" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1495" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1495" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1496" spans="1:4">
+      <c r="A1496" s="80"/>
+      <c r="B1496" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1496" s="84" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1496" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1497" spans="1:4">
+      <c r="A1497" s="80"/>
+      <c r="B1497" s="2" t="s">
+        <v>497</v>
+      </c>
+      <c r="C1497" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1497" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1498" spans="1:4">
+      <c r="A1498" s="85"/>
+      <c r="B1498" s="2" t="s">
+        <v>498</v>
+      </c>
+      <c r="C1498" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1498" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1500" spans="1:4">
+      <c r="A1500" s="86">
+        <v>46066</v>
+      </c>
+      <c r="B1500" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1500" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1500" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1501" spans="1:4">
+      <c r="A1501" s="80"/>
+      <c r="B1501" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1501" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1501" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1502" spans="1:4">
+      <c r="A1502" s="80"/>
+      <c r="B1502" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1502" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1502" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1503" spans="1:4">
+      <c r="A1503" s="80"/>
+      <c r="B1503" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1503" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1503" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1504" spans="1:4">
+      <c r="A1504" s="80"/>
+      <c r="B1504" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1504" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1504" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1505" spans="1:4">
+      <c r="A1505" s="80"/>
+      <c r="B1505" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1505" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1505" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1506" spans="1:4">
+      <c r="A1506" s="80"/>
+      <c r="B1506" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1506" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1506" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1507" spans="1:4">
+      <c r="A1507" s="80"/>
+      <c r="B1507" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1507" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1507" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1508" spans="1:4">
+      <c r="A1508" s="80"/>
+      <c r="B1508" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1508" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1508" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1509" spans="1:4">
+      <c r="A1509" s="80"/>
+      <c r="B1509" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1509" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1509" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1510" spans="1:4">
+      <c r="A1510" s="80"/>
+      <c r="B1510" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1510" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1510" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1511" spans="1:4">
+      <c r="A1511" s="80"/>
+      <c r="B1511" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1511" s="93" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1511" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1512" spans="1:4">
+      <c r="A1512" s="80"/>
+      <c r="B1512" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1512" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1512" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1513" spans="1:4">
+      <c r="A1513" s="80"/>
+      <c r="B1513" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1513" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1513" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1514" spans="1:4">
+      <c r="A1514" s="85"/>
+      <c r="B1514" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1514" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1514" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1516" spans="1:4">
+      <c r="A1516" s="86">
+        <v>46067</v>
+      </c>
+      <c r="B1516" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1516" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1516" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1517" spans="1:4">
+      <c r="A1517" s="80"/>
+      <c r="B1517" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1517" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1517" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1518" spans="1:4">
+      <c r="A1518" s="80"/>
+      <c r="B1518" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1518" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1518" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1519" spans="1:4">
+      <c r="A1519" s="80"/>
+      <c r="B1519" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1519" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1519" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1520" spans="1:4">
+      <c r="A1520" s="80"/>
+      <c r="B1520" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1520" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1520" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1521" spans="1:4">
+      <c r="A1521" s="80"/>
+      <c r="B1521" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1521" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1521" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1522" spans="1:4">
+      <c r="A1522" s="80"/>
+      <c r="B1522" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1522" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1522" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1523" spans="1:4">
+      <c r="A1523" s="80"/>
+      <c r="B1523" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1523" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1523" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1524" spans="1:4">
+      <c r="A1524" s="80"/>
+      <c r="B1524" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1524" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1524" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1525" spans="1:4">
+      <c r="A1525" s="80"/>
+      <c r="B1525" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1525" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1525" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1526" spans="1:4">
+      <c r="A1526" s="80"/>
+      <c r="B1526" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1526" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1526" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1527" spans="1:4">
+      <c r="A1527" s="80"/>
+      <c r="B1527" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1527" s="93" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1527" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1528" spans="1:4">
+      <c r="A1528" s="80"/>
+      <c r="B1528" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1528" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1528" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1529" spans="1:4">
+      <c r="A1529" s="80"/>
+      <c r="B1529" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1529" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1529" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1530" spans="1:4">
+      <c r="A1530" s="85"/>
+      <c r="B1530" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1530" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1530" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1532" spans="1:4">
+      <c r="A1532" s="86">
+        <v>46067</v>
+      </c>
+      <c r="B1532" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1532" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1532" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1533" spans="1:4">
+      <c r="A1533" s="80"/>
+      <c r="B1533" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1533" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1533" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1534" spans="1:4">
+      <c r="A1534" s="80"/>
+      <c r="B1534" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1534" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1534" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1535" spans="1:4">
+      <c r="A1535" s="80"/>
+      <c r="B1535" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1535" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1535" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1536" spans="1:4">
+      <c r="A1536" s="80"/>
+      <c r="B1536" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1536" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1536" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1537" spans="1:4">
+      <c r="A1537" s="80"/>
+      <c r="B1537" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1537" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1537" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1538" spans="1:4">
+      <c r="A1538" s="80"/>
+      <c r="B1538" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1538" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1538" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1539" spans="1:4">
+      <c r="A1539" s="80"/>
+      <c r="B1539" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1539" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1539" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1540" spans="1:4">
+      <c r="A1540" s="80"/>
+      <c r="B1540" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1540" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1540" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1541" spans="1:4">
+      <c r="A1541" s="80"/>
+      <c r="B1541" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1541" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1541" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1542" spans="1:4">
+      <c r="A1542" s="80"/>
+      <c r="B1542" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1542" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1542" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1543" spans="1:4">
+      <c r="A1543" s="80"/>
+      <c r="B1543" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1543" s="93" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1543" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1544" spans="1:4">
+      <c r="A1544" s="80"/>
+      <c r="B1544" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1544" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1544" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1545" spans="1:4">
+      <c r="A1545" s="80"/>
+      <c r="B1545" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1545" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1545" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1546" spans="1:4">
+      <c r="A1546" s="80"/>
+      <c r="B1546" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1546" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1546" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1547" spans="1:4">
+      <c r="A1547" s="85"/>
+      <c r="B1547" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C1547" s="111" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1547" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1549" spans="1:4">
+      <c r="A1549" s="112">
+        <v>46070</v>
+      </c>
+      <c r="B1549" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1549" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1549" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1550" spans="1:4">
+      <c r="A1550" s="113"/>
+      <c r="B1550" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1550" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1550" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1551" spans="1:4">
+      <c r="A1551" s="113"/>
+      <c r="B1551" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1551" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1551" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1552" spans="1:4">
+      <c r="A1552" s="113"/>
+      <c r="B1552" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1552" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1552" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1553" spans="1:4">
+      <c r="A1553" s="113"/>
+      <c r="B1553" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1553" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1553" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1554" spans="1:4">
+      <c r="A1554" s="113"/>
+      <c r="B1554" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1554" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1554" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1555" spans="1:4">
+      <c r="A1555" s="113"/>
+      <c r="B1555" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1555" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1555" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1556" spans="1:4">
+      <c r="A1556" s="113"/>
+      <c r="B1556" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1556" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1556" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1557" spans="1:4">
+      <c r="A1557" s="113"/>
+      <c r="B1557" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1557" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1557" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1558" spans="1:4">
+      <c r="A1558" s="113"/>
+      <c r="B1558" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1558" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1558" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1559" spans="1:4">
+      <c r="A1559" s="113"/>
+      <c r="B1559" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1559" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1559" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1560" spans="1:4">
+      <c r="A1560" s="113"/>
+      <c r="B1560" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1560" s="93" t="s">
+        <v>501</v>
+      </c>
+      <c r="D1560" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1561" spans="1:4">
+      <c r="A1561" s="113"/>
+      <c r="B1561" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1561" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1561" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1562" spans="1:4">
+      <c r="A1562" s="113"/>
+      <c r="B1562" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1562" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1562" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1563" spans="1:4">
+      <c r="A1563" s="113"/>
+      <c r="B1563" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1563" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1563" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1564" spans="1:4">
+      <c r="A1564" s="113"/>
+      <c r="B1564" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="C1564" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1564" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1565" spans="1:4">
+      <c r="A1565" s="113"/>
+      <c r="B1565" s="114" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1565" s="115" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1565" s="116" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1566" spans="1:4">
+      <c r="A1566" s="113"/>
+      <c r="B1566" s="114" t="s">
+        <v>508</v>
+      </c>
+      <c r="C1566" s="115" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1566" s="116" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:4">
+      <c r="A1567" s="117"/>
+      <c r="B1567" s="114" t="s">
+        <v>509</v>
+      </c>
+      <c r="C1567" s="115" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1567" s="116" t="s">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="91">
+  <mergeCells count="99">
     <mergeCell ref="A2:A15"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A23:A30"/>
@@ -20258,6 +21744,14 @@
     <mergeCell ref="A1401:A1412"/>
     <mergeCell ref="A1414:A1428"/>
     <mergeCell ref="A1430:A1443"/>
+    <mergeCell ref="A1445:A1458"/>
+    <mergeCell ref="A1460:A1468"/>
+    <mergeCell ref="A1470:A1483"/>
+    <mergeCell ref="A1485:A1498"/>
+    <mergeCell ref="A1500:A1514"/>
+    <mergeCell ref="A1516:A1530"/>
+    <mergeCell ref="A1532:A1547"/>
+    <mergeCell ref="A1549:A1567"/>
     <mergeCell ref="D24:D25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -20295,32 +21789,32 @@
   <sheetData>
     <row r="1" s="27" customFormat="1" spans="1:10">
       <c r="A1" s="35" t="s">
-        <v>491</v>
+        <v>510</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>492</v>
+        <v>511</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>493</v>
+        <v>512</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>494</v>
+        <v>513</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>495</v>
+        <v>514</v>
       </c>
       <c r="F1" s="52" t="s">
-        <v>496</v>
+        <v>515</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>497</v>
+        <v>516</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>498</v>
+        <v>517</v>
       </c>
       <c r="I1" s="66"/>
       <c r="J1" s="67" t="s">
-        <v>499</v>
+        <v>518</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -20328,10 +21822,10 @@
         <v>45954</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>501</v>
+        <v>520</v>
       </c>
       <c r="D2" s="39">
         <v>16</v>
@@ -20358,10 +21852,10 @@
         <v>45956</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>502</v>
+        <v>521</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>503</v>
+        <v>522</v>
       </c>
       <c r="D3" s="43">
         <v>5.7</v>
@@ -20377,16 +21871,16 @@
       <c r="G3" s="42"/>
       <c r="H3" s="56"/>
       <c r="J3" s="67" t="s">
-        <v>504</v>
+        <v>523</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="40"/>
       <c r="B4" s="41" t="s">
-        <v>505</v>
+        <v>524</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>506</v>
+        <v>525</v>
       </c>
       <c r="D4" s="43">
         <v>3.5</v>
@@ -20405,10 +21899,10 @@
     <row r="5" s="28" customFormat="1" spans="1:10">
       <c r="A5" s="40"/>
       <c r="B5" s="41" t="s">
-        <v>507</v>
+        <v>526</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>508</v>
+        <v>527</v>
       </c>
       <c r="D5" s="43">
         <v>5.8</v>
@@ -20422,7 +21916,7 @@
       <c r="H5" s="56"/>
       <c r="I5" s="27"/>
       <c r="J5" s="67" t="s">
-        <v>509</v>
+        <v>528</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -20430,10 +21924,10 @@
         <v>45957</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>510</v>
+        <v>529</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>511</v>
+        <v>530</v>
       </c>
       <c r="D6" s="39">
         <v>23</v>
@@ -20458,10 +21952,10 @@
         <v>45958</v>
       </c>
       <c r="B7" s="41" t="s">
-        <v>512</v>
+        <v>531</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>513</v>
+        <v>532</v>
       </c>
       <c r="D7" s="43">
         <v>23</v>
@@ -20478,16 +21972,16 @@
       <c r="H7" s="56"/>
       <c r="I7" s="27"/>
       <c r="J7" s="67" t="s">
-        <v>514</v>
+        <v>533</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="40"/>
       <c r="B8" s="41" t="s">
-        <v>515</v>
+        <v>534</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>516</v>
+        <v>535</v>
       </c>
       <c r="D8" s="43">
         <v>5.3</v>
@@ -20509,10 +22003,10 @@
         <v>45959</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>517</v>
+        <v>536</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>518</v>
+        <v>537</v>
       </c>
       <c r="D9" s="39">
         <v>30</v>
@@ -20529,7 +22023,7 @@
       <c r="H9" s="56"/>
       <c r="I9" s="27"/>
       <c r="J9" s="67" t="s">
-        <v>519</v>
+        <v>538</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -20537,10 +22031,10 @@
         <v>45960</v>
       </c>
       <c r="B10" s="41" t="s">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>521</v>
+        <v>540</v>
       </c>
       <c r="D10" s="43">
         <v>30</v>
@@ -20562,10 +22056,10 @@
     <row r="11" spans="1:10">
       <c r="A11" s="40"/>
       <c r="B11" s="41" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>523</v>
+        <v>542</v>
       </c>
       <c r="D11" s="43">
         <v>11</v>
@@ -20579,16 +22073,16 @@
       <c r="H11" s="56"/>
       <c r="I11" s="27"/>
       <c r="J11" s="70" t="s">
-        <v>524</v>
+        <v>543</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="40"/>
       <c r="B12" s="41" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>526</v>
+        <v>545</v>
       </c>
       <c r="D12" s="43">
         <v>12</v>
@@ -20608,10 +22102,10 @@
     <row r="13" spans="1:10">
       <c r="A13" s="40"/>
       <c r="B13" s="41" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>527</v>
+        <v>546</v>
       </c>
       <c r="D13" s="43">
         <v>11</v>
@@ -20625,16 +22119,16 @@
       <c r="H13" s="56"/>
       <c r="I13" s="27"/>
       <c r="J13" s="70" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="40"/>
       <c r="B14" s="41" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
       <c r="C14" s="42" t="s">
-        <v>529</v>
+        <v>548</v>
       </c>
       <c r="D14" s="43">
         <v>12</v>
@@ -20654,10 +22148,10 @@
     <row r="15" spans="1:10">
       <c r="A15" s="40"/>
       <c r="B15" s="41" t="s">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="D15" s="43">
         <v>13.2</v>
@@ -20671,7 +22165,7 @@
       <c r="H15" s="56"/>
       <c r="I15" s="27"/>
       <c r="J15" s="70" t="s">
-        <v>532</v>
+        <v>551</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -20679,10 +22173,10 @@
         <v>45961</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>533</v>
+        <v>552</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>534</v>
+        <v>553</v>
       </c>
       <c r="D16" s="39">
         <v>11.4</v>
@@ -20705,10 +22199,10 @@
     <row r="17" spans="1:10">
       <c r="A17" s="36"/>
       <c r="B17" s="37" t="s">
-        <v>535</v>
+        <v>554</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="D17" s="39">
         <v>12.6</v>
@@ -20722,7 +22216,7 @@
       <c r="H17" s="56"/>
       <c r="I17" s="27"/>
       <c r="J17" s="71" t="s">
-        <v>537</v>
+        <v>556</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -20730,10 +22224,10 @@
         <v>45964</v>
       </c>
       <c r="B18" s="41" t="s">
-        <v>538</v>
+        <v>557</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>539</v>
+        <v>558</v>
       </c>
       <c r="D18" s="43">
         <v>24</v>
@@ -20756,10 +22250,10 @@
     <row r="19" spans="1:9">
       <c r="A19" s="40"/>
       <c r="B19" s="41" t="s">
-        <v>540</v>
+        <v>559</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>541</v>
+        <v>560</v>
       </c>
       <c r="D19" s="43">
         <v>13.4</v>
@@ -20778,10 +22272,10 @@
         <v>45966</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>542</v>
+        <v>561</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>543</v>
+        <v>562</v>
       </c>
       <c r="D20" s="47">
         <v>8.2</v>
@@ -20800,10 +22294,10 @@
     <row r="21" spans="1:9">
       <c r="A21" s="44"/>
       <c r="B21" s="45" t="s">
-        <v>544</v>
+        <v>563</v>
       </c>
       <c r="C21" s="46" t="s">
-        <v>545</v>
+        <v>564</v>
       </c>
       <c r="D21" s="47">
         <v>27</v>
@@ -20820,10 +22314,10 @@
     <row r="22" spans="1:8">
       <c r="A22" s="44"/>
       <c r="B22" s="45" t="s">
-        <v>546</v>
+        <v>565</v>
       </c>
       <c r="C22" s="46" t="s">
-        <v>547</v>
+        <v>566</v>
       </c>
       <c r="D22" s="47">
         <v>22</v>
@@ -20841,10 +22335,10 @@
         <v>45967</v>
       </c>
       <c r="B23" s="42" t="s">
-        <v>538</v>
+        <v>557</v>
       </c>
       <c r="C23" s="42" t="s">
-        <v>548</v>
+        <v>567</v>
       </c>
       <c r="D23" s="43">
         <v>24</v>
@@ -20863,10 +22357,10 @@
     <row r="24" spans="1:8">
       <c r="A24" s="40"/>
       <c r="B24" s="41" t="s">
-        <v>515</v>
+        <v>534</v>
       </c>
       <c r="C24" s="42" t="s">
-        <v>549</v>
+        <v>568</v>
       </c>
       <c r="D24" s="43">
         <v>12</v>
@@ -20884,10 +22378,10 @@
         <v>45969</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>550</v>
+        <v>569</v>
       </c>
       <c r="C25" s="46" t="s">
-        <v>551</v>
+        <v>570</v>
       </c>
       <c r="D25" s="47">
         <v>12.4</v>
@@ -20908,10 +22402,10 @@
         <v>45971</v>
       </c>
       <c r="B26" s="41" t="s">
-        <v>552</v>
+        <v>571</v>
       </c>
       <c r="C26" s="42" t="s">
-        <v>553</v>
+        <v>572</v>
       </c>
       <c r="D26" s="43">
         <v>15.8</v>
@@ -20932,10 +22426,10 @@
         <v>45972</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>535</v>
+        <v>554</v>
       </c>
       <c r="C27" s="46" t="s">
-        <v>554</v>
+        <v>573</v>
       </c>
       <c r="D27" s="47">
         <v>13</v>
@@ -20956,10 +22450,10 @@
         <v>45974</v>
       </c>
       <c r="B28" s="41" t="s">
-        <v>555</v>
+        <v>574</v>
       </c>
       <c r="C28" s="42" t="s">
-        <v>556</v>
+        <v>575</v>
       </c>
       <c r="D28" s="43">
         <v>15</v>
@@ -20978,10 +22472,10 @@
     <row r="29" spans="1:8">
       <c r="A29" s="40"/>
       <c r="B29" s="41" t="s">
-        <v>557</v>
+        <v>576</v>
       </c>
       <c r="C29" s="42" t="s">
-        <v>558</v>
+        <v>577</v>
       </c>
       <c r="D29" s="43">
         <v>20</v>
@@ -20999,10 +22493,10 @@
         <v>45979</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>559</v>
+        <v>578</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>560</v>
+        <v>579</v>
       </c>
       <c r="D30" s="47">
         <v>12</v>
@@ -21023,10 +22517,10 @@
         <v>45980</v>
       </c>
       <c r="B31" s="41" t="s">
-        <v>533</v>
+        <v>552</v>
       </c>
       <c r="C31" s="42" t="s">
-        <v>561</v>
+        <v>580</v>
       </c>
       <c r="D31" s="43">
         <v>10.9</v>
@@ -21045,10 +22539,10 @@
     <row r="32" spans="1:8">
       <c r="A32" s="40"/>
       <c r="B32" s="41" t="s">
-        <v>562</v>
+        <v>581</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>563</v>
+        <v>582</v>
       </c>
       <c r="D32" s="43">
         <v>18</v>
@@ -21066,10 +22560,10 @@
         <v>45982</v>
       </c>
       <c r="B33" s="45" t="s">
-        <v>564</v>
+        <v>583</v>
       </c>
       <c r="C33" s="46" t="s">
-        <v>565</v>
+        <v>584</v>
       </c>
       <c r="D33" s="47">
         <v>3.6</v>
@@ -21088,10 +22582,10 @@
     <row r="34" spans="1:8">
       <c r="A34" s="44"/>
       <c r="B34" s="45" t="s">
-        <v>566</v>
+        <v>585</v>
       </c>
       <c r="C34" s="46" t="s">
-        <v>567</v>
+        <v>586</v>
       </c>
       <c r="D34" s="47">
         <v>16</v>
@@ -21107,10 +22601,10 @@
     <row r="35" spans="1:8">
       <c r="A35" s="44"/>
       <c r="B35" s="45" t="s">
-        <v>568</v>
+        <v>587</v>
       </c>
       <c r="C35" s="46" t="s">
-        <v>569</v>
+        <v>588</v>
       </c>
       <c r="D35" s="47">
         <v>13.4</v>
@@ -21126,10 +22620,10 @@
     <row r="36" spans="1:8">
       <c r="A36" s="44"/>
       <c r="B36" s="45" t="s">
-        <v>559</v>
+        <v>578</v>
       </c>
       <c r="C36" s="46" t="s">
-        <v>570</v>
+        <v>589</v>
       </c>
       <c r="D36" s="47">
         <v>12</v>
@@ -21145,10 +22639,10 @@
     <row r="37" spans="1:8">
       <c r="A37" s="44"/>
       <c r="B37" s="45" t="s">
-        <v>571</v>
+        <v>590</v>
       </c>
       <c r="C37" s="46" t="s">
-        <v>572</v>
+        <v>591</v>
       </c>
       <c r="D37" s="47">
         <v>16.4</v>
@@ -21166,10 +22660,10 @@
         <v>45983</v>
       </c>
       <c r="B38" s="41" t="s">
-        <v>573</v>
+        <v>592</v>
       </c>
       <c r="C38" s="42" t="s">
-        <v>574</v>
+        <v>593</v>
       </c>
       <c r="D38" s="43">
         <v>14</v>
@@ -21190,10 +22684,10 @@
         <v>45987</v>
       </c>
       <c r="B39" s="45" t="s">
-        <v>575</v>
+        <v>594</v>
       </c>
       <c r="C39" s="46" t="s">
-        <v>576</v>
+        <v>595</v>
       </c>
       <c r="D39" s="47">
         <v>16</v>
@@ -21212,10 +22706,10 @@
     <row r="40" spans="1:8">
       <c r="A40" s="44"/>
       <c r="B40" s="45" t="s">
-        <v>577</v>
+        <v>596</v>
       </c>
       <c r="C40" s="46" t="s">
-        <v>578</v>
+        <v>597</v>
       </c>
       <c r="D40" s="47">
         <v>12.4</v>
@@ -21233,10 +22727,10 @@
         <v>45988</v>
       </c>
       <c r="B41" s="41" t="s">
-        <v>579</v>
+        <v>598</v>
       </c>
       <c r="C41" s="42" t="s">
-        <v>580</v>
+        <v>599</v>
       </c>
       <c r="D41" s="43">
         <v>22</v>
@@ -21255,10 +22749,10 @@
     <row r="42" spans="1:8">
       <c r="A42" s="40"/>
       <c r="B42" s="41" t="s">
-        <v>581</v>
+        <v>600</v>
       </c>
       <c r="C42" s="42" t="s">
-        <v>582</v>
+        <v>601</v>
       </c>
       <c r="D42" s="43">
         <v>13.2</v>
@@ -21276,10 +22770,10 @@
         <v>45990</v>
       </c>
       <c r="B43" s="45" t="s">
-        <v>583</v>
+        <v>602</v>
       </c>
       <c r="C43" s="46" t="s">
-        <v>584</v>
+        <v>603</v>
       </c>
       <c r="D43" s="47">
         <v>15.2</v>
@@ -21300,10 +22794,10 @@
         <v>45992</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>585</v>
+        <v>604</v>
       </c>
       <c r="C44" s="42" t="s">
-        <v>586</v>
+        <v>605</v>
       </c>
       <c r="D44" s="43">
         <v>2.8</v>
@@ -21322,10 +22816,10 @@
     <row r="45" spans="1:8">
       <c r="A45" s="40"/>
       <c r="B45" s="41" t="s">
-        <v>587</v>
+        <v>606</v>
       </c>
       <c r="C45" s="42" t="s">
-        <v>588</v>
+        <v>607</v>
       </c>
       <c r="D45" s="43">
         <v>16</v>
@@ -21343,10 +22837,10 @@
         <v>45995</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>589</v>
+        <v>608</v>
       </c>
       <c r="C46" s="38" t="s">
-        <v>590</v>
+        <v>609</v>
       </c>
       <c r="D46" s="39">
         <v>68</v>
@@ -21367,10 +22861,10 @@
         <v>45996</v>
       </c>
       <c r="B47" s="41" t="s">
-        <v>591</v>
+        <v>610</v>
       </c>
       <c r="C47" s="42" t="s">
-        <v>592</v>
+        <v>611</v>
       </c>
       <c r="D47" s="43">
         <v>25</v>
@@ -21389,10 +22883,10 @@
     <row r="48" spans="1:8">
       <c r="A48" s="40"/>
       <c r="B48" s="41" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="C48" s="42" t="s">
-        <v>594</v>
+        <v>613</v>
       </c>
       <c r="D48" s="43">
         <v>24</v>
@@ -21410,10 +22904,10 @@
         <v>45997</v>
       </c>
       <c r="B49" s="37" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="C49" s="38" t="s">
-        <v>595</v>
+        <v>614</v>
       </c>
       <c r="D49" s="39">
         <v>12</v>
@@ -21434,10 +22928,10 @@
         <v>45999</v>
       </c>
       <c r="B50" s="41" t="s">
-        <v>596</v>
+        <v>615</v>
       </c>
       <c r="C50" s="42" t="s">
-        <v>597</v>
+        <v>616</v>
       </c>
       <c r="D50" s="43">
         <v>9.9</v>
@@ -21456,10 +22950,10 @@
     <row r="51" spans="1:8">
       <c r="A51" s="40"/>
       <c r="B51" s="41" t="s">
-        <v>568</v>
+        <v>587</v>
       </c>
       <c r="C51" s="42" t="s">
-        <v>598</v>
+        <v>617</v>
       </c>
       <c r="D51" s="43">
         <v>12.8</v>
@@ -21477,10 +22971,10 @@
         <v>46000</v>
       </c>
       <c r="B52" s="37" t="s">
-        <v>599</v>
+        <v>618</v>
       </c>
       <c r="C52" s="38" t="s">
-        <v>600</v>
+        <v>619</v>
       </c>
       <c r="D52" s="39">
         <v>24</v>
@@ -21499,10 +22993,10 @@
     <row r="53" spans="1:8">
       <c r="A53" s="36"/>
       <c r="B53" s="37" t="s">
-        <v>601</v>
+        <v>620</v>
       </c>
       <c r="C53" s="38" t="s">
-        <v>602</v>
+        <v>621</v>
       </c>
       <c r="D53" s="39">
         <v>12.2</v>
@@ -21518,10 +23012,10 @@
     <row r="54" spans="1:8">
       <c r="A54" s="36"/>
       <c r="B54" s="37" t="s">
-        <v>568</v>
+        <v>587</v>
       </c>
       <c r="C54" s="38" t="s">
-        <v>603</v>
+        <v>622</v>
       </c>
       <c r="D54" s="39">
         <v>13.4</v>
@@ -21539,10 +23033,10 @@
         <v>46001</v>
       </c>
       <c r="B55" s="41" t="s">
-        <v>583</v>
+        <v>602</v>
       </c>
       <c r="C55" s="42" t="s">
-        <v>604</v>
+        <v>623</v>
       </c>
       <c r="D55" s="43">
         <v>15.2</v>
@@ -21563,10 +23057,10 @@
         <v>46002</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>593</v>
+        <v>612</v>
       </c>
       <c r="C56" s="38" t="s">
-        <v>605</v>
+        <v>624</v>
       </c>
       <c r="D56" s="39">
         <v>12</v>
@@ -21584,10 +23078,10 @@
         <v>46010</v>
       </c>
       <c r="B57" s="49" t="s">
-        <v>606</v>
+        <v>625</v>
       </c>
       <c r="C57" s="50" t="s">
-        <v>607</v>
+        <v>626</v>
       </c>
       <c r="D57" s="51">
         <v>3.4</v>
@@ -21608,10 +23102,10 @@
         <v>46016</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>608</v>
+        <v>627</v>
       </c>
       <c r="C58" s="38" t="s">
-        <v>609</v>
+        <v>628</v>
       </c>
       <c r="D58" s="39">
         <v>14</v>
@@ -21632,10 +23126,10 @@
         <v>46016</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="C59" s="38" t="s">
-        <v>610</v>
+        <v>629</v>
       </c>
       <c r="D59" s="39">
         <v>22</v>
@@ -21713,31 +23207,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>611</v>
+        <v>630</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>612</v>
+        <v>631</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>613</v>
+        <v>632</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>614</v>
+        <v>633</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>615</v>
+        <v>634</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>616</v>
+        <v>635</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>617</v>
+        <v>636</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>618</v>
+        <v>637</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>619</v>
+        <v>638</v>
       </c>
     </row>
     <row r="2" ht="126.7" customHeight="1" spans="1:10">
@@ -21745,16 +23239,16 @@
         <v>45967</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>620</v>
+        <v>639</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>621</v>
+        <v>640</v>
       </c>
       <c r="D2" s="15">
         <v>3</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>622</v>
+        <v>641</v>
       </c>
       <c r="F2" s="22"/>
       <c r="G2" s="23">
@@ -21769,7 +23263,7 @@
         <v>846000</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>623</v>
+        <v>642</v>
       </c>
     </row>
     <row r="3" ht="43" customHeight="1" spans="1:10">
@@ -21942,21 +23436,21 @@
   <sheetData>
     <row r="1" spans="2:3">
       <c r="B1" s="1" t="s">
-        <v>624</v>
+        <v>643</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="1" t="s">
-        <v>625</v>
+        <v>644</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>626</v>
+        <v>645</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
-        <v>627</v>
+        <v>646</v>
       </c>
       <c r="C3" s="2">
         <v>6699</v>
@@ -21964,7 +23458,7 @@
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="2" t="s">
-        <v>628</v>
+        <v>647</v>
       </c>
       <c r="C4" s="2">
         <v>2323</v>
@@ -21972,7 +23466,7 @@
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="2" t="s">
-        <v>629</v>
+        <v>648</v>
       </c>
       <c r="C5" s="2">
         <v>8899</v>
@@ -21980,7 +23474,7 @@
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="2" t="s">
-        <v>630</v>
+        <v>649</v>
       </c>
       <c r="C6" s="2">
         <v>5656</v>
@@ -21988,7 +23482,7 @@
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="2" t="s">
-        <v>631</v>
+        <v>650</v>
       </c>
       <c r="C7" s="2">
         <v>7744</v>
@@ -21996,7 +23490,7 @@
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="2" t="s">
-        <v>632</v>
+        <v>651</v>
       </c>
       <c r="C8" s="2">
         <v>4545</v>
@@ -22004,7 +23498,7 @@
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="2" t="s">
-        <v>633</v>
+        <v>652</v>
       </c>
       <c r="C9" s="2">
         <v>2525</v>
@@ -22012,7 +23506,7 @@
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="2" t="s">
-        <v>634</v>
+        <v>653</v>
       </c>
       <c r="C10" s="2">
         <v>3636</v>

</xml_diff>

<commit_message>
Friday 27 feb 14:53
updated
</commit_message>
<xml_diff>
--- a/Daily Activities.xlsx
+++ b/Daily Activities.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11260" windowHeight="17020"/>
+    <workbookView windowWidth="16360" windowHeight="18640"/>
   </bookViews>
   <sheets>
     <sheet name="Daily Acitivies &amp; Checklists" sheetId="26" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4539" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4974" uniqueCount="671">
   <si>
     <t>DATE</t>
   </si>
@@ -1556,10 +1556,61 @@
     <t>Purchase fruit knife for bar</t>
   </si>
   <si>
+    <t>Nachos 1 kg matang</t>
+  </si>
+  <si>
     <t>Tortilla matang 6 bungkus</t>
   </si>
   <si>
     <t>Purchase fox glue 2 pack</t>
+  </si>
+  <si>
+    <t>ALREADY APPROVED ON LEMESY</t>
+  </si>
+  <si>
+    <t>Purchase flies trapper for bar</t>
+  </si>
+  <si>
+    <t>Already bought 3 paint sample</t>
+  </si>
+  <si>
+    <t>Purchase rubber band for kitchen labelling</t>
+  </si>
+  <si>
+    <t>Purchase stickers for kitchen labelling</t>
+  </si>
+  <si>
+    <t>Find 25" monitor w AIO that has windows OS 2nd 4 million budget</t>
+  </si>
+  <si>
+    <t>Buy another plant to replace the dead one</t>
+  </si>
+  <si>
+    <t>Already put printing waiting for lemesy payment</t>
+  </si>
+  <si>
+    <t>Already got another sampling jade jazz</t>
+  </si>
+  <si>
+    <t>Posted on lemesy</t>
+  </si>
+  <si>
+    <t>Purchase bar lamp, and kitchen exhaust lamp</t>
+  </si>
+  <si>
+    <t>Purchase screws for the trolley</t>
+  </si>
+  <si>
+    <t>Purchase another 70 L of fresh milk</t>
+  </si>
+  <si>
+    <t>Already paid on Tokopedia</t>
+  </si>
+  <si>
+    <t>Will post another reference</t>
+  </si>
+  <si>
+    <t>Purchase 2 pcs of zigger for bar</t>
   </si>
   <si>
     <t>Date</t>
@@ -2208,7 +2259,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2272,6 +2323,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2653,7 +2710,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -2677,16 +2734,16 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="14" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -2695,89 +2752,89 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="42" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="118">
+  <cellXfs count="123">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -3120,6 +3177,9 @@
     <xf numFmtId="180" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -3129,8 +3189,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="180" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -3802,7 +3874,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K1567"/>
+  <dimension ref="A1:K1720"/>
   <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12.859375" style="72"/>
@@ -21423,7 +21495,7 @@
       </c>
     </row>
     <row r="1549" spans="1:4">
-      <c r="A1549" s="112">
+      <c r="A1549" s="86">
         <v>46070</v>
       </c>
       <c r="B1549" s="106" t="s">
@@ -21437,7 +21509,7 @@
       </c>
     </row>
     <row r="1550" spans="1:4">
-      <c r="A1550" s="113"/>
+      <c r="A1550" s="80"/>
       <c r="B1550" s="106" t="s">
         <v>287</v>
       </c>
@@ -21449,7 +21521,7 @@
       </c>
     </row>
     <row r="1551" spans="1:4">
-      <c r="A1551" s="113"/>
+      <c r="A1551" s="80"/>
       <c r="B1551" s="106" t="s">
         <v>303</v>
       </c>
@@ -21461,7 +21533,7 @@
       </c>
     </row>
     <row r="1552" spans="1:4">
-      <c r="A1552" s="113"/>
+      <c r="A1552" s="80"/>
       <c r="B1552" s="106" t="s">
         <v>434</v>
       </c>
@@ -21473,7 +21545,7 @@
       </c>
     </row>
     <row r="1553" spans="1:4">
-      <c r="A1553" s="113"/>
+      <c r="A1553" s="80"/>
       <c r="B1553" s="106" t="s">
         <v>450</v>
       </c>
@@ -21485,7 +21557,7 @@
       </c>
     </row>
     <row r="1554" spans="1:4">
-      <c r="A1554" s="113"/>
+      <c r="A1554" s="80"/>
       <c r="B1554" s="106" t="s">
         <v>467</v>
       </c>
@@ -21497,7 +21569,7 @@
       </c>
     </row>
     <row r="1555" spans="1:4">
-      <c r="A1555" s="113"/>
+      <c r="A1555" s="80"/>
       <c r="B1555" s="2" t="s">
         <v>490</v>
       </c>
@@ -21509,7 +21581,7 @@
       </c>
     </row>
     <row r="1556" spans="1:4">
-      <c r="A1556" s="113"/>
+      <c r="A1556" s="80"/>
       <c r="B1556" s="2" t="s">
         <v>494</v>
       </c>
@@ -21521,7 +21593,7 @@
       </c>
     </row>
     <row r="1557" spans="1:4">
-      <c r="A1557" s="113"/>
+      <c r="A1557" s="80"/>
       <c r="B1557" s="2" t="s">
         <v>495</v>
       </c>
@@ -21533,7 +21605,7 @@
       </c>
     </row>
     <row r="1558" spans="1:4">
-      <c r="A1558" s="113"/>
+      <c r="A1558" s="80"/>
       <c r="B1558" s="2" t="s">
         <v>496</v>
       </c>
@@ -21545,7 +21617,7 @@
       </c>
     </row>
     <row r="1559" spans="1:4">
-      <c r="A1559" s="113"/>
+      <c r="A1559" s="80"/>
       <c r="B1559" s="2" t="s">
         <v>499</v>
       </c>
@@ -21557,7 +21629,7 @@
       </c>
     </row>
     <row r="1560" spans="1:4">
-      <c r="A1560" s="113"/>
+      <c r="A1560" s="80"/>
       <c r="B1560" s="2" t="s">
         <v>500</v>
       </c>
@@ -21569,7 +21641,7 @@
       </c>
     </row>
     <row r="1561" spans="1:4">
-      <c r="A1561" s="113"/>
+      <c r="A1561" s="80"/>
       <c r="B1561" s="2" t="s">
         <v>502</v>
       </c>
@@ -21581,7 +21653,7 @@
       </c>
     </row>
     <row r="1562" spans="1:4">
-      <c r="A1562" s="113"/>
+      <c r="A1562" s="80"/>
       <c r="B1562" s="2" t="s">
         <v>503</v>
       </c>
@@ -21593,7 +21665,7 @@
       </c>
     </row>
     <row r="1563" spans="1:4">
-      <c r="A1563" s="113"/>
+      <c r="A1563" s="80"/>
       <c r="B1563" s="2" t="s">
         <v>504</v>
       </c>
@@ -21605,7 +21677,7 @@
       </c>
     </row>
     <row r="1564" spans="1:4">
-      <c r="A1564" s="113"/>
+      <c r="A1564" s="80"/>
       <c r="B1564" s="2" t="s">
         <v>507</v>
       </c>
@@ -21617,43 +21689,1799 @@
       </c>
     </row>
     <row r="1565" spans="1:4">
-      <c r="A1565" s="113"/>
-      <c r="B1565" s="114" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1565" s="115" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1565" s="116" t="s">
+      <c r="A1565" s="80"/>
+      <c r="B1565" s="2" t="s">
+        <v>508</v>
+      </c>
+      <c r="C1565" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1565" s="1" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="1566" spans="1:4">
-      <c r="A1566" s="113"/>
-      <c r="B1566" s="114" t="s">
+      <c r="A1566" s="80"/>
+      <c r="B1566" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C1566" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1566" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1567" spans="1:4">
+      <c r="A1567" s="85"/>
+      <c r="B1567" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1567" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1567" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1569" spans="1:4">
+      <c r="A1569" s="112">
+        <v>46071</v>
+      </c>
+      <c r="B1569" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1569" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1569" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1570" spans="1:4">
+      <c r="A1570" s="113"/>
+      <c r="B1570" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1570" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1570" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1571" spans="1:4">
+      <c r="A1571" s="113"/>
+      <c r="B1571" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1571" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1571" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1572" spans="1:4">
+      <c r="A1572" s="113"/>
+      <c r="B1572" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1572" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1572" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1573" spans="1:4">
+      <c r="A1573" s="113"/>
+      <c r="B1573" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1573" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1573" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1574" spans="1:4">
+      <c r="A1574" s="113"/>
+      <c r="B1574" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1574" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1574" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1575" spans="1:4">
+      <c r="A1575" s="113"/>
+      <c r="B1575" s="2" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1575" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1575" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1576" spans="1:4">
+      <c r="A1576" s="113"/>
+      <c r="B1576" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1576" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1576" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1577" spans="1:4">
+      <c r="A1577" s="113"/>
+      <c r="B1577" s="2" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1577" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1577" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1578" spans="1:4">
+      <c r="A1578" s="113"/>
+      <c r="B1578" s="2" t="s">
+        <v>496</v>
+      </c>
+      <c r="C1578" s="84" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1578" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1579" spans="1:4">
+      <c r="A1579" s="113"/>
+      <c r="B1579" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1579" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1579" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1580" spans="1:4">
+      <c r="A1580" s="113"/>
+      <c r="B1580" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1580" s="93" t="s">
+        <v>511</v>
+      </c>
+      <c r="D1580" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1581" spans="1:4">
+      <c r="A1581" s="113"/>
+      <c r="B1581" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1581" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1581" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1582" spans="1:4">
+      <c r="A1582" s="113"/>
+      <c r="B1582" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1582" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1582" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1583" spans="1:4">
+      <c r="A1583" s="113"/>
+      <c r="B1583" s="2" t="s">
+        <v>504</v>
+      </c>
+      <c r="C1583" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1583" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1584" spans="1:4">
+      <c r="A1584" s="113"/>
+      <c r="B1584" s="2" t="s">
         <v>508</v>
       </c>
-      <c r="C1566" s="115" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1566" s="116" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="1567" spans="1:4">
-      <c r="A1567" s="117"/>
-      <c r="B1567" s="114" t="s">
+      <c r="C1584" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1584" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1585" spans="1:4">
+      <c r="A1585" s="113"/>
+      <c r="B1585" s="2" t="s">
         <v>509</v>
       </c>
-      <c r="C1567" s="115" t="s">
-        <v>97</v>
-      </c>
-      <c r="D1567" s="116" t="s">
+      <c r="C1585" s="84" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1585" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1586" spans="1:4">
+      <c r="A1586" s="113"/>
+      <c r="B1586" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1586" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1586" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1587" spans="1:4">
+      <c r="A1587" s="114"/>
+      <c r="B1587" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1587" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1587" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1589" spans="1:4">
+      <c r="A1589" s="112">
+        <v>46072</v>
+      </c>
+      <c r="B1589" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1589" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1589" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1590" spans="1:4">
+      <c r="A1590" s="113"/>
+      <c r="B1590" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1590" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1590" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1591" spans="1:4">
+      <c r="A1591" s="113"/>
+      <c r="B1591" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1591" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1591" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1592" spans="1:4">
+      <c r="A1592" s="113"/>
+      <c r="B1592" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1592" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1592" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1593" spans="1:4">
+      <c r="A1593" s="113"/>
+      <c r="B1593" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1593" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1593" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1594" spans="1:4">
+      <c r="A1594" s="113"/>
+      <c r="B1594" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1594" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1594" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1595" spans="1:4">
+      <c r="A1595" s="113"/>
+      <c r="B1595" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1595" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1595" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1596" spans="1:4">
+      <c r="A1596" s="113"/>
+      <c r="B1596" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1596" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1596" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1597" spans="1:4">
+      <c r="A1597" s="113"/>
+      <c r="B1597" s="118" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1597" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1597" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1598" spans="1:4">
+      <c r="A1598" s="113"/>
+      <c r="B1598" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1598" s="93" t="s">
+        <v>513</v>
+      </c>
+      <c r="D1598" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1599" spans="1:4">
+      <c r="A1599" s="113"/>
+      <c r="B1599" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1599" s="93" t="s">
+        <v>511</v>
+      </c>
+      <c r="D1599" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1600" spans="1:4">
+      <c r="A1600" s="113"/>
+      <c r="B1600" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1600" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1600" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1601" spans="1:4">
+      <c r="A1601" s="113"/>
+      <c r="B1601" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1601" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1601" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1602" spans="1:4">
+      <c r="A1602" s="113"/>
+      <c r="B1602" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1602" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1602" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1603" spans="1:4">
+      <c r="A1603" s="113"/>
+      <c r="B1603" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1603" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1603" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1604" spans="1:4">
+      <c r="A1604" s="113"/>
+      <c r="B1604" s="115" t="s">
+        <v>514</v>
+      </c>
+      <c r="C1604" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1604" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1605" spans="1:4">
+      <c r="A1605" s="113"/>
+      <c r="B1605" s="115" t="s">
+        <v>515</v>
+      </c>
+      <c r="C1605" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1605" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1606" spans="1:4">
+      <c r="A1606" s="113"/>
+      <c r="B1606" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1606" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1606" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1607" spans="1:4">
+      <c r="A1607" s="114"/>
+      <c r="B1607" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1607" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1607" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1609" spans="1:4">
+      <c r="A1609" s="112">
+        <v>46073</v>
+      </c>
+      <c r="B1609" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1609" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1609" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1610" spans="1:4">
+      <c r="A1610" s="113"/>
+      <c r="B1610" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1610" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1610" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1611" spans="1:4">
+      <c r="A1611" s="113"/>
+      <c r="B1611" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1611" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1611" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1612" spans="1:4">
+      <c r="A1612" s="113"/>
+      <c r="B1612" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1612" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1612" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1613" spans="1:4">
+      <c r="A1613" s="113"/>
+      <c r="B1613" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1613" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1613" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1614" spans="1:4">
+      <c r="A1614" s="113"/>
+      <c r="B1614" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1614" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1614" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1615" spans="1:4">
+      <c r="A1615" s="113"/>
+      <c r="B1615" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1615" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1615" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1616" spans="1:4">
+      <c r="A1616" s="113"/>
+      <c r="B1616" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1616" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1616" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1617" spans="1:4">
+      <c r="A1617" s="113"/>
+      <c r="B1617" s="118" t="s">
+        <v>495</v>
+      </c>
+      <c r="C1617" s="110" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1617" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1618" spans="1:4">
+      <c r="A1618" s="113"/>
+      <c r="B1618" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1618" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1618" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1619" spans="1:4">
+      <c r="A1619" s="113"/>
+      <c r="B1619" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1619" s="93" t="s">
+        <v>511</v>
+      </c>
+      <c r="D1619" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1620" spans="1:4">
+      <c r="A1620" s="113"/>
+      <c r="B1620" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1620" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1620" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1621" spans="1:4">
+      <c r="A1621" s="113"/>
+      <c r="B1621" s="2" t="s">
+        <v>503</v>
+      </c>
+      <c r="C1621" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1621" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1622" spans="1:4">
+      <c r="A1622" s="113"/>
+      <c r="B1622" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1622" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1622" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1623" spans="1:4">
+      <c r="A1623" s="113"/>
+      <c r="B1623" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1623" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1623" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1624" spans="1:4">
+      <c r="A1624" s="113"/>
+      <c r="B1624" s="115" t="s">
+        <v>514</v>
+      </c>
+      <c r="C1624" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1624" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1625" spans="1:4">
+      <c r="A1625" s="113"/>
+      <c r="B1625" s="115" t="s">
+        <v>515</v>
+      </c>
+      <c r="C1625" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1625" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1626" spans="1:4">
+      <c r="A1626" s="113"/>
+      <c r="B1626" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1626" s="116" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1626" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1627" spans="1:4">
+      <c r="A1627" s="114"/>
+      <c r="B1627" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1627" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1627" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1629" spans="1:4">
+      <c r="A1629" s="112">
+        <v>46074</v>
+      </c>
+      <c r="B1629" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1629" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1629" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1630" spans="1:4">
+      <c r="A1630" s="113"/>
+      <c r="B1630" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1630" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1630" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1631" spans="1:4">
+      <c r="A1631" s="113"/>
+      <c r="B1631" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1631" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1631" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1632" spans="1:4">
+      <c r="A1632" s="113"/>
+      <c r="B1632" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1632" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1632" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1633" spans="1:4">
+      <c r="A1633" s="113"/>
+      <c r="B1633" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1633" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1633" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1634" spans="1:4">
+      <c r="A1634" s="113"/>
+      <c r="B1634" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1634" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1634" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1635" spans="1:4">
+      <c r="A1635" s="113"/>
+      <c r="B1635" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1635" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1635" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1636" spans="1:4">
+      <c r="A1636" s="113"/>
+      <c r="B1636" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1636" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1636" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1637" spans="1:4">
+      <c r="A1637" s="113"/>
+      <c r="B1637" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1637" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1637" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1638" spans="1:4">
+      <c r="A1638" s="113"/>
+      <c r="B1638" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1638" s="93" t="s">
+        <v>511</v>
+      </c>
+      <c r="D1638" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1639" spans="1:4">
+      <c r="A1639" s="113"/>
+      <c r="B1639" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1639" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1639" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1640" spans="1:4">
+      <c r="A1640" s="113"/>
+      <c r="B1640" s="118" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1640" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1640" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1641" spans="1:4">
+      <c r="A1641" s="113"/>
+      <c r="B1641" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1641" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1641" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1642" spans="1:4">
+      <c r="A1642" s="113"/>
+      <c r="B1642" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1642" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1642" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1643" spans="1:4">
+      <c r="A1643" s="113"/>
+      <c r="B1643" s="115" t="s">
+        <v>514</v>
+      </c>
+      <c r="C1643" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1643" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1644" spans="1:4">
+      <c r="A1644" s="113"/>
+      <c r="B1644" s="115" t="s">
+        <v>515</v>
+      </c>
+      <c r="C1644" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1644" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1645" spans="1:4">
+      <c r="A1645" s="113"/>
+      <c r="B1645" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1645" s="116" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1645" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1646" spans="1:4">
+      <c r="A1646" s="113"/>
+      <c r="B1646" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1646" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1646" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1647" spans="1:4">
+      <c r="A1647" s="114"/>
+      <c r="B1647" s="119" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1647" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1647" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1649" spans="1:4">
+      <c r="A1649" s="112">
+        <v>46075</v>
+      </c>
+      <c r="B1649" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1649" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1649" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1650" spans="1:4">
+      <c r="A1650" s="113"/>
+      <c r="B1650" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1650" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1650" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1651" spans="1:4">
+      <c r="A1651" s="113"/>
+      <c r="B1651" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1651" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1651" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1652" spans="1:4">
+      <c r="A1652" s="113"/>
+      <c r="B1652" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1652" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1652" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1653" spans="1:4">
+      <c r="A1653" s="113"/>
+      <c r="B1653" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1653" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1653" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1654" spans="1:4">
+      <c r="A1654" s="113"/>
+      <c r="B1654" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1654" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1654" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1655" spans="1:4">
+      <c r="A1655" s="113"/>
+      <c r="B1655" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1655" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1655" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1656" spans="1:4">
+      <c r="A1656" s="113"/>
+      <c r="B1656" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1656" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1656" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1657" spans="1:4">
+      <c r="A1657" s="113"/>
+      <c r="B1657" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1657" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1657" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1658" spans="1:4">
+      <c r="A1658" s="113"/>
+      <c r="B1658" s="2" t="s">
+        <v>500</v>
+      </c>
+      <c r="C1658" s="84" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1658" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1659" spans="1:4">
+      <c r="A1659" s="113"/>
+      <c r="B1659" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1659" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1659" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1660" spans="1:4">
+      <c r="A1660" s="113"/>
+      <c r="B1660" s="118" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1660" s="93" t="s">
+        <v>506</v>
+      </c>
+      <c r="D1660" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1661" spans="1:4">
+      <c r="A1661" s="113"/>
+      <c r="B1661" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1661" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1661" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1662" spans="1:4">
+      <c r="A1662" s="113"/>
+      <c r="B1662" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1662" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1662" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1663" spans="1:4">
+      <c r="A1663" s="113"/>
+      <c r="B1663" s="115" t="s">
+        <v>514</v>
+      </c>
+      <c r="C1663" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1663" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1664" spans="1:4">
+      <c r="A1664" s="113"/>
+      <c r="B1664" s="115" t="s">
+        <v>515</v>
+      </c>
+      <c r="C1664" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1664" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1665" spans="1:4">
+      <c r="A1665" s="113"/>
+      <c r="B1665" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1665" s="116" t="s">
+        <v>520</v>
+      </c>
+      <c r="D1665" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1666" spans="1:4">
+      <c r="A1666" s="113"/>
+      <c r="B1666" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1666" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1666" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1667" spans="1:4">
+      <c r="A1667" s="113"/>
+      <c r="B1667" s="119" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1667" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1667" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1668" spans="1:4">
+      <c r="A1668" s="114"/>
+      <c r="B1668" s="115" t="s">
+        <v>523</v>
+      </c>
+      <c r="C1668" s="120" t="s">
+        <v>171</v>
+      </c>
+      <c r="D1668" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1670" spans="1:4">
+      <c r="A1670" s="112">
+        <v>46077</v>
+      </c>
+      <c r="B1670" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1670" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1670" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1671" spans="1:4">
+      <c r="A1671" s="113"/>
+      <c r="B1671" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1671" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1671" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1672" spans="1:4">
+      <c r="A1672" s="113"/>
+      <c r="B1672" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1672" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1672" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1673" spans="1:4">
+      <c r="A1673" s="113"/>
+      <c r="B1673" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1673" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1673" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1674" spans="1:4">
+      <c r="A1674" s="113"/>
+      <c r="B1674" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1674" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1674" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1675" spans="1:4">
+      <c r="A1675" s="113"/>
+      <c r="B1675" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1675" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1675" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1676" spans="1:4">
+      <c r="A1676" s="113"/>
+      <c r="B1676" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1676" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1676" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1677" spans="1:4">
+      <c r="A1677" s="113"/>
+      <c r="B1677" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1677" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1677" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1678" spans="1:4">
+      <c r="A1678" s="113"/>
+      <c r="B1678" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1678" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1678" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1679" spans="1:4">
+      <c r="A1679" s="113"/>
+      <c r="B1679" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1679" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1679" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1680" spans="1:4">
+      <c r="A1680" s="113"/>
+      <c r="B1680" s="118" t="s">
+        <v>521</v>
+      </c>
+      <c r="C1680" s="121" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1680" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1681" spans="1:4">
+      <c r="A1681" s="113"/>
+      <c r="B1681" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1681" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1681" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1682" spans="1:4">
+      <c r="A1682" s="113"/>
+      <c r="B1682" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1682" s="116" t="s">
+        <v>524</v>
+      </c>
+      <c r="D1682" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1683" spans="1:4">
+      <c r="A1683" s="113"/>
+      <c r="B1683" s="115" t="s">
+        <v>514</v>
+      </c>
+      <c r="C1683" s="122" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1683" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1684" spans="1:4">
+      <c r="A1684" s="113"/>
+      <c r="B1684" s="115" t="s">
+        <v>515</v>
+      </c>
+      <c r="C1684" s="122" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1684" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1685" spans="1:4">
+      <c r="A1685" s="113"/>
+      <c r="B1685" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1685" s="116" t="s">
+        <v>525</v>
+      </c>
+      <c r="D1685" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1686" spans="1:4">
+      <c r="A1686" s="113"/>
+      <c r="B1686" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1686" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1686" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1687" spans="1:4">
+      <c r="A1687" s="113"/>
+      <c r="B1687" s="119" t="s">
+        <v>522</v>
+      </c>
+      <c r="C1687" s="122" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1687" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1688" spans="1:4">
+      <c r="A1688" s="114"/>
+      <c r="B1688" s="115" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1688" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1688" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1690" spans="1:4">
+      <c r="A1690" s="112">
+        <v>46078</v>
+      </c>
+      <c r="B1690" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1690" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1690" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1691" spans="1:4">
+      <c r="A1691" s="113"/>
+      <c r="B1691" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1691" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1691" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1692" spans="1:4">
+      <c r="A1692" s="113"/>
+      <c r="B1692" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1692" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1692" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1693" spans="1:4">
+      <c r="A1693" s="113"/>
+      <c r="B1693" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1693" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1693" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1694" spans="1:4">
+      <c r="A1694" s="113"/>
+      <c r="B1694" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1694" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1694" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1695" spans="1:4">
+      <c r="A1695" s="113"/>
+      <c r="B1695" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1695" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1695" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1696" spans="1:4">
+      <c r="A1696" s="113"/>
+      <c r="B1696" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1696" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1696" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1697" spans="1:4">
+      <c r="A1697" s="113"/>
+      <c r="B1697" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1697" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1697" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1698" spans="1:4">
+      <c r="A1698" s="113"/>
+      <c r="B1698" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1698" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1698" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1699" spans="1:4">
+      <c r="A1699" s="113"/>
+      <c r="B1699" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1699" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1699" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1700" spans="1:4">
+      <c r="A1700" s="113"/>
+      <c r="B1700" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1700" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1700" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1701" spans="1:4">
+      <c r="A1701" s="113"/>
+      <c r="B1701" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1701" s="116" t="s">
+        <v>524</v>
+      </c>
+      <c r="D1701" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1702" spans="1:4">
+      <c r="A1702" s="113"/>
+      <c r="B1702" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1702" s="116" t="s">
+        <v>525</v>
+      </c>
+      <c r="D1702" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1703" spans="1:4">
+      <c r="A1703" s="113"/>
+      <c r="B1703" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1703" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1703" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1704" spans="1:4">
+      <c r="A1704" s="114"/>
+      <c r="B1704" s="115" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1704" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1704" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1706" spans="1:4">
+      <c r="A1706" s="112">
+        <v>46079</v>
+      </c>
+      <c r="B1706" s="106" t="s">
+        <v>259</v>
+      </c>
+      <c r="C1706" s="78" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1706" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1707" spans="1:4">
+      <c r="A1707" s="113"/>
+      <c r="B1707" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="C1707" s="93" t="s">
+        <v>292</v>
+      </c>
+      <c r="D1707" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1708" spans="1:4">
+      <c r="A1708" s="113"/>
+      <c r="B1708" s="106" t="s">
+        <v>303</v>
+      </c>
+      <c r="C1708" s="93" t="s">
+        <v>308</v>
+      </c>
+      <c r="D1708" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1709" spans="1:4">
+      <c r="A1709" s="113"/>
+      <c r="B1709" s="106" t="s">
+        <v>434</v>
+      </c>
+      <c r="C1709" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1709" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1710" spans="1:4">
+      <c r="A1710" s="113"/>
+      <c r="B1710" s="106" t="s">
+        <v>450</v>
+      </c>
+      <c r="C1710" s="93" t="s">
+        <v>463</v>
+      </c>
+      <c r="D1710" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1711" spans="1:4">
+      <c r="A1711" s="113"/>
+      <c r="B1711" s="106" t="s">
+        <v>467</v>
+      </c>
+      <c r="C1711" s="93" t="s">
+        <v>472</v>
+      </c>
+      <c r="D1711" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1712" spans="1:4">
+      <c r="A1712" s="113"/>
+      <c r="B1712" s="118" t="s">
+        <v>490</v>
+      </c>
+      <c r="C1712" s="93" t="s">
+        <v>518</v>
+      </c>
+      <c r="D1712" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1713" spans="1:4">
+      <c r="A1713" s="113"/>
+      <c r="B1713" s="2" t="s">
+        <v>494</v>
+      </c>
+      <c r="C1713" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1713" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1714" spans="1:4">
+      <c r="A1714" s="113"/>
+      <c r="B1714" s="2" t="s">
+        <v>499</v>
+      </c>
+      <c r="C1714" s="93" t="s">
+        <v>519</v>
+      </c>
+      <c r="D1714" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1715" spans="1:4">
+      <c r="A1715" s="113"/>
+      <c r="B1715" s="2" t="s">
+        <v>502</v>
+      </c>
+      <c r="C1715" s="93" t="s">
+        <v>505</v>
+      </c>
+      <c r="D1715" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1716" spans="1:4">
+      <c r="A1716" s="113"/>
+      <c r="B1716" s="2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C1716" s="93" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1716" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1717" spans="1:4">
+      <c r="A1717" s="113"/>
+      <c r="B1717" s="115" t="s">
+        <v>512</v>
+      </c>
+      <c r="C1717" s="116" t="s">
+        <v>524</v>
+      </c>
+      <c r="D1717" s="117" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1718" spans="1:4">
+      <c r="A1718" s="113"/>
+      <c r="B1718" s="115" t="s">
+        <v>516</v>
+      </c>
+      <c r="C1718" s="116" t="s">
+        <v>525</v>
+      </c>
+      <c r="D1718" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1719" spans="1:4">
+      <c r="A1719" s="113"/>
+      <c r="B1719" s="115" t="s">
+        <v>517</v>
+      </c>
+      <c r="C1719" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1719" s="117" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="1720" spans="1:4">
+      <c r="A1720" s="114"/>
+      <c r="B1720" s="115" t="s">
+        <v>526</v>
+      </c>
+      <c r="C1720" s="116" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1720" s="117" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="99">
+  <mergeCells count="107">
     <mergeCell ref="A2:A15"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A23:A30"/>
@@ -21752,6 +23580,14 @@
     <mergeCell ref="A1516:A1530"/>
     <mergeCell ref="A1532:A1547"/>
     <mergeCell ref="A1549:A1567"/>
+    <mergeCell ref="A1569:A1587"/>
+    <mergeCell ref="A1589:A1607"/>
+    <mergeCell ref="A1609:A1627"/>
+    <mergeCell ref="A1629:A1647"/>
+    <mergeCell ref="A1649:A1668"/>
+    <mergeCell ref="A1670:A1688"/>
+    <mergeCell ref="A1690:A1704"/>
+    <mergeCell ref="A1706:A1720"/>
     <mergeCell ref="D24:D25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -21789,32 +23625,32 @@
   <sheetData>
     <row r="1" s="27" customFormat="1" spans="1:10">
       <c r="A1" s="35" t="s">
-        <v>510</v>
+        <v>527</v>
       </c>
       <c r="B1" s="35" t="s">
-        <v>511</v>
+        <v>528</v>
       </c>
       <c r="C1" s="35" t="s">
-        <v>512</v>
+        <v>529</v>
       </c>
       <c r="D1" s="35" t="s">
-        <v>513</v>
+        <v>530</v>
       </c>
       <c r="E1" s="35" t="s">
-        <v>514</v>
+        <v>531</v>
       </c>
       <c r="F1" s="52" t="s">
-        <v>515</v>
+        <v>532</v>
       </c>
       <c r="G1" s="35" t="s">
-        <v>516</v>
+        <v>533</v>
       </c>
       <c r="H1" s="35" t="s">
-        <v>517</v>
+        <v>534</v>
       </c>
       <c r="I1" s="66"/>
       <c r="J1" s="67" t="s">
-        <v>518</v>
+        <v>535</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -21822,10 +23658,10 @@
         <v>45954</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>519</v>
+        <v>536</v>
       </c>
       <c r="C2" s="38" t="s">
-        <v>520</v>
+        <v>537</v>
       </c>
       <c r="D2" s="39">
         <v>16</v>
@@ -21852,10 +23688,10 @@
         <v>45956</v>
       </c>
       <c r="B3" s="41" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
       <c r="C3" s="42" t="s">
-        <v>522</v>
+        <v>539</v>
       </c>
       <c r="D3" s="43">
         <v>5.7</v>
@@ -21871,16 +23707,16 @@
       <c r="G3" s="42"/>
       <c r="H3" s="56"/>
       <c r="J3" s="67" t="s">
-        <v>523</v>
+        <v>540</v>
       </c>
     </row>
     <row r="4" spans="1:10">
       <c r="A4" s="40"/>
       <c r="B4" s="41" t="s">
-        <v>524</v>
+        <v>541</v>
       </c>
       <c r="C4" s="42" t="s">
-        <v>525</v>
+        <v>542</v>
       </c>
       <c r="D4" s="43">
         <v>3.5</v>
@@ -21899,10 +23735,10 @@
     <row r="5" s="28" customFormat="1" spans="1:10">
       <c r="A5" s="40"/>
       <c r="B5" s="41" t="s">
-        <v>526</v>
+        <v>543</v>
       </c>
       <c r="C5" s="42" t="s">
-        <v>527</v>
+        <v>544</v>
       </c>
       <c r="D5" s="43">
         <v>5.8</v>
@@ -21916,7 +23752,7 @@
       <c r="H5" s="56"/>
       <c r="I5" s="27"/>
       <c r="J5" s="67" t="s">
-        <v>528</v>
+        <v>545</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -21924,10 +23760,10 @@
         <v>45957</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>529</v>
+        <v>546</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>530</v>
+        <v>547</v>
       </c>
       <c r="D6" s="39">
         <v>23</v>
@@ -21952,10 +23788,10 @@
         <v>45958</v>
       </c>
       <c r="B7" s="41" t="s">
-        <v>531</v>
+        <v>548</v>
       </c>
       <c r="C7" s="42" t="s">
-        <v>532</v>
+        <v>549</v>
       </c>
       <c r="D7" s="43">
         <v>23</v>
@@ -21972,16 +23808,16 @@
       <c r="H7" s="56"/>
       <c r="I7" s="27"/>
       <c r="J7" s="67" t="s">
-        <v>533</v>
+        <v>550</v>
       </c>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="40"/>
       <c r="B8" s="41" t="s">
-        <v>534</v>
+        <v>551</v>
       </c>
       <c r="C8" s="42" t="s">
-        <v>535</v>
+        <v>552</v>
       </c>
       <c r="D8" s="43">
         <v>5.3</v>
@@ -22003,10 +23839,10 @@
         <v>45959</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>536</v>
+        <v>553</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>537</v>
+        <v>554</v>
       </c>
       <c r="D9" s="39">
         <v>30</v>
@@ -22023,7 +23859,7 @@
       <c r="H9" s="56"/>
       <c r="I9" s="27"/>
       <c r="J9" s="67" t="s">
-        <v>538</v>
+        <v>555</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -22031,10 +23867,10 @@
         <v>45960</v>
       </c>
       <c r="B10" s="41" t="s">
-        <v>539</v>
+        <v>556</v>
       </c>
       <c r="C10" s="42" t="s">
-        <v>540</v>
+        <v>557</v>
       </c>
       <c r="D10" s="43">
         <v>30</v>
@@ -22056,10 +23892,10 @@
     <row r="11" spans="1:10">
       <c r="A11" s="40"/>
       <c r="B11" s="41" t="s">
-        <v>541</v>
+        <v>558</v>
       </c>
       <c r="C11" s="42" t="s">
-        <v>542</v>
+        <v>559</v>
       </c>
       <c r="D11" s="43">
         <v>11</v>
@@ -22073,16 +23909,16 @@
       <c r="H11" s="56"/>
       <c r="I11" s="27"/>
       <c r="J11" s="70" t="s">
-        <v>543</v>
+        <v>560</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="40"/>
       <c r="B12" s="41" t="s">
-        <v>544</v>
+        <v>561</v>
       </c>
       <c r="C12" s="42" t="s">
-        <v>545</v>
+        <v>562</v>
       </c>
       <c r="D12" s="43">
         <v>12</v>
@@ -22102,10 +23938,10 @@
     <row r="13" spans="1:10">
       <c r="A13" s="40"/>
       <c r="B13" s="41" t="s">
-        <v>541</v>
+        <v>558</v>
       </c>
       <c r="C13" s="42" t="s">
-        <v>546</v>
+        <v>563</v>
       </c>
       <c r="D13" s="43">
         <v>11</v>
@@ -22119,16 +23955,16 @@
       <c r="H13" s="56"/>
       <c r="I13" s="27"/>
       <c r="J13" s="70" t="s">
-        <v>547</v>
+        <v>564</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="40"/>
       <c r="B14" s="41" t="s">
-        <v>544</v>
+        <v>561</v>
       </c>
       <c r="C14" s="42" t="s">
-        <v>548</v>
+        <v>565</v>
       </c>
       <c r="D14" s="43">
         <v>12</v>
@@ -22148,10 +23984,10 @@
     <row r="15" spans="1:10">
       <c r="A15" s="40"/>
       <c r="B15" s="41" t="s">
-        <v>549</v>
+        <v>566</v>
       </c>
       <c r="C15" s="42" t="s">
-        <v>550</v>
+        <v>567</v>
       </c>
       <c r="D15" s="43">
         <v>13.2</v>
@@ -22165,7 +24001,7 @@
       <c r="H15" s="56"/>
       <c r="I15" s="27"/>
       <c r="J15" s="70" t="s">
-        <v>551</v>
+        <v>568</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -22173,10 +24009,10 @@
         <v>45961</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
       <c r="C16" s="38" t="s">
-        <v>553</v>
+        <v>570</v>
       </c>
       <c r="D16" s="39">
         <v>11.4</v>
@@ -22199,10 +24035,10 @@
     <row r="17" spans="1:10">
       <c r="A17" s="36"/>
       <c r="B17" s="37" t="s">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>555</v>
+        <v>572</v>
       </c>
       <c r="D17" s="39">
         <v>12.6</v>
@@ -22216,7 +24052,7 @@
       <c r="H17" s="56"/>
       <c r="I17" s="27"/>
       <c r="J17" s="71" t="s">
-        <v>556</v>
+        <v>573</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -22224,10 +24060,10 @@
         <v>45964</v>
       </c>
       <c r="B18" s="41" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="C18" s="42" t="s">
-        <v>558</v>
+        <v>575</v>
       </c>
       <c r="D18" s="43">
         <v>24</v>
@@ -22250,10 +24086,10 @@
     <row r="19" spans="1:9">
       <c r="A19" s="40"/>
       <c r="B19" s="41" t="s">
-        <v>559</v>
+        <v>576</v>
       </c>
       <c r="C19" s="42" t="s">
-        <v>560</v>
+        <v>577</v>
       </c>
       <c r="D19" s="43">
         <v>13.4</v>
@@ -22272,10 +24108,10 @@
         <v>45966</v>
       </c>
       <c r="B20" s="45" t="s">
-        <v>561</v>
+        <v>578</v>
       </c>
       <c r="C20" s="46" t="s">
-        <v>562</v>
+        <v>579</v>
       </c>
       <c r="D20" s="47">
         <v>8.2</v>
@@ -22294,10 +24130,10 @@
     <row r="21" spans="1:9">
       <c r="A21" s="44"/>
       <c r="B21" s="45" t="s">
-        <v>563</v>
+        <v>580</v>
       </c>
       <c r="C21" s="46" t="s">
-        <v>564</v>
+        <v>581</v>
       </c>
       <c r="D21" s="47">
         <v>27</v>
@@ -22314,10 +24150,10 @@
     <row r="22" spans="1:8">
       <c r="A22" s="44"/>
       <c r="B22" s="45" t="s">
-        <v>565</v>
+        <v>582</v>
       </c>
       <c r="C22" s="46" t="s">
-        <v>566</v>
+        <v>583</v>
       </c>
       <c r="D22" s="47">
         <v>22</v>
@@ -22335,10 +24171,10 @@
         <v>45967</v>
       </c>
       <c r="B23" s="42" t="s">
-        <v>557</v>
+        <v>574</v>
       </c>
       <c r="C23" s="42" t="s">
-        <v>567</v>
+        <v>584</v>
       </c>
       <c r="D23" s="43">
         <v>24</v>
@@ -22357,10 +24193,10 @@
     <row r="24" spans="1:8">
       <c r="A24" s="40"/>
       <c r="B24" s="41" t="s">
-        <v>534</v>
+        <v>551</v>
       </c>
       <c r="C24" s="42" t="s">
-        <v>568</v>
+        <v>585</v>
       </c>
       <c r="D24" s="43">
         <v>12</v>
@@ -22378,10 +24214,10 @@
         <v>45969</v>
       </c>
       <c r="B25" s="45" t="s">
-        <v>569</v>
+        <v>586</v>
       </c>
       <c r="C25" s="46" t="s">
-        <v>570</v>
+        <v>587</v>
       </c>
       <c r="D25" s="47">
         <v>12.4</v>
@@ -22402,10 +24238,10 @@
         <v>45971</v>
       </c>
       <c r="B26" s="41" t="s">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="C26" s="42" t="s">
-        <v>572</v>
+        <v>589</v>
       </c>
       <c r="D26" s="43">
         <v>15.8</v>
@@ -22426,10 +24262,10 @@
         <v>45972</v>
       </c>
       <c r="B27" s="45" t="s">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="C27" s="46" t="s">
-        <v>573</v>
+        <v>590</v>
       </c>
       <c r="D27" s="47">
         <v>13</v>
@@ -22450,10 +24286,10 @@
         <v>45974</v>
       </c>
       <c r="B28" s="41" t="s">
-        <v>574</v>
+        <v>591</v>
       </c>
       <c r="C28" s="42" t="s">
-        <v>575</v>
+        <v>592</v>
       </c>
       <c r="D28" s="43">
         <v>15</v>
@@ -22472,10 +24308,10 @@
     <row r="29" spans="1:8">
       <c r="A29" s="40"/>
       <c r="B29" s="41" t="s">
-        <v>576</v>
+        <v>593</v>
       </c>
       <c r="C29" s="42" t="s">
-        <v>577</v>
+        <v>594</v>
       </c>
       <c r="D29" s="43">
         <v>20</v>
@@ -22493,10 +24329,10 @@
         <v>45979</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="C30" s="46" t="s">
-        <v>579</v>
+        <v>596</v>
       </c>
       <c r="D30" s="47">
         <v>12</v>
@@ -22517,10 +24353,10 @@
         <v>45980</v>
       </c>
       <c r="B31" s="41" t="s">
-        <v>552</v>
+        <v>569</v>
       </c>
       <c r="C31" s="42" t="s">
-        <v>580</v>
+        <v>597</v>
       </c>
       <c r="D31" s="43">
         <v>10.9</v>
@@ -22539,10 +24375,10 @@
     <row r="32" spans="1:8">
       <c r="A32" s="40"/>
       <c r="B32" s="41" t="s">
-        <v>581</v>
+        <v>598</v>
       </c>
       <c r="C32" s="42" t="s">
-        <v>582</v>
+        <v>599</v>
       </c>
       <c r="D32" s="43">
         <v>18</v>
@@ -22560,10 +24396,10 @@
         <v>45982</v>
       </c>
       <c r="B33" s="45" t="s">
-        <v>583</v>
+        <v>600</v>
       </c>
       <c r="C33" s="46" t="s">
-        <v>584</v>
+        <v>601</v>
       </c>
       <c r="D33" s="47">
         <v>3.6</v>
@@ -22582,10 +24418,10 @@
     <row r="34" spans="1:8">
       <c r="A34" s="44"/>
       <c r="B34" s="45" t="s">
-        <v>585</v>
+        <v>602</v>
       </c>
       <c r="C34" s="46" t="s">
-        <v>586</v>
+        <v>603</v>
       </c>
       <c r="D34" s="47">
         <v>16</v>
@@ -22601,10 +24437,10 @@
     <row r="35" spans="1:8">
       <c r="A35" s="44"/>
       <c r="B35" s="45" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="C35" s="46" t="s">
-        <v>588</v>
+        <v>605</v>
       </c>
       <c r="D35" s="47">
         <v>13.4</v>
@@ -22620,10 +24456,10 @@
     <row r="36" spans="1:8">
       <c r="A36" s="44"/>
       <c r="B36" s="45" t="s">
-        <v>578</v>
+        <v>595</v>
       </c>
       <c r="C36" s="46" t="s">
-        <v>589</v>
+        <v>606</v>
       </c>
       <c r="D36" s="47">
         <v>12</v>
@@ -22639,10 +24475,10 @@
     <row r="37" spans="1:8">
       <c r="A37" s="44"/>
       <c r="B37" s="45" t="s">
-        <v>590</v>
+        <v>607</v>
       </c>
       <c r="C37" s="46" t="s">
-        <v>591</v>
+        <v>608</v>
       </c>
       <c r="D37" s="47">
         <v>16.4</v>
@@ -22660,10 +24496,10 @@
         <v>45983</v>
       </c>
       <c r="B38" s="41" t="s">
-        <v>592</v>
+        <v>609</v>
       </c>
       <c r="C38" s="42" t="s">
-        <v>593</v>
+        <v>610</v>
       </c>
       <c r="D38" s="43">
         <v>14</v>
@@ -22684,10 +24520,10 @@
         <v>45987</v>
       </c>
       <c r="B39" s="45" t="s">
-        <v>594</v>
+        <v>611</v>
       </c>
       <c r="C39" s="46" t="s">
-        <v>595</v>
+        <v>612</v>
       </c>
       <c r="D39" s="47">
         <v>16</v>
@@ -22706,10 +24542,10 @@
     <row r="40" spans="1:8">
       <c r="A40" s="44"/>
       <c r="B40" s="45" t="s">
-        <v>596</v>
+        <v>613</v>
       </c>
       <c r="C40" s="46" t="s">
-        <v>597</v>
+        <v>614</v>
       </c>
       <c r="D40" s="47">
         <v>12.4</v>
@@ -22727,10 +24563,10 @@
         <v>45988</v>
       </c>
       <c r="B41" s="41" t="s">
-        <v>598</v>
+        <v>615</v>
       </c>
       <c r="C41" s="42" t="s">
-        <v>599</v>
+        <v>616</v>
       </c>
       <c r="D41" s="43">
         <v>22</v>
@@ -22749,10 +24585,10 @@
     <row r="42" spans="1:8">
       <c r="A42" s="40"/>
       <c r="B42" s="41" t="s">
-        <v>600</v>
+        <v>617</v>
       </c>
       <c r="C42" s="42" t="s">
-        <v>601</v>
+        <v>618</v>
       </c>
       <c r="D42" s="43">
         <v>13.2</v>
@@ -22770,10 +24606,10 @@
         <v>45990</v>
       </c>
       <c r="B43" s="45" t="s">
-        <v>602</v>
+        <v>619</v>
       </c>
       <c r="C43" s="46" t="s">
-        <v>603</v>
+        <v>620</v>
       </c>
       <c r="D43" s="47">
         <v>15.2</v>
@@ -22794,10 +24630,10 @@
         <v>45992</v>
       </c>
       <c r="B44" s="41" t="s">
-        <v>604</v>
+        <v>621</v>
       </c>
       <c r="C44" s="42" t="s">
-        <v>605</v>
+        <v>622</v>
       </c>
       <c r="D44" s="43">
         <v>2.8</v>
@@ -22816,10 +24652,10 @@
     <row r="45" spans="1:8">
       <c r="A45" s="40"/>
       <c r="B45" s="41" t="s">
-        <v>606</v>
+        <v>623</v>
       </c>
       <c r="C45" s="42" t="s">
-        <v>607</v>
+        <v>624</v>
       </c>
       <c r="D45" s="43">
         <v>16</v>
@@ -22837,10 +24673,10 @@
         <v>45995</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>608</v>
+        <v>625</v>
       </c>
       <c r="C46" s="38" t="s">
-        <v>609</v>
+        <v>626</v>
       </c>
       <c r="D46" s="39">
         <v>68</v>
@@ -22861,10 +24697,10 @@
         <v>45996</v>
       </c>
       <c r="B47" s="41" t="s">
-        <v>610</v>
+        <v>627</v>
       </c>
       <c r="C47" s="42" t="s">
-        <v>611</v>
+        <v>628</v>
       </c>
       <c r="D47" s="43">
         <v>25</v>
@@ -22883,10 +24719,10 @@
     <row r="48" spans="1:8">
       <c r="A48" s="40"/>
       <c r="B48" s="41" t="s">
-        <v>612</v>
+        <v>629</v>
       </c>
       <c r="C48" s="42" t="s">
-        <v>613</v>
+        <v>630</v>
       </c>
       <c r="D48" s="43">
         <v>24</v>
@@ -22904,10 +24740,10 @@
         <v>45997</v>
       </c>
       <c r="B49" s="37" t="s">
-        <v>612</v>
+        <v>629</v>
       </c>
       <c r="C49" s="38" t="s">
-        <v>614</v>
+        <v>631</v>
       </c>
       <c r="D49" s="39">
         <v>12</v>
@@ -22928,10 +24764,10 @@
         <v>45999</v>
       </c>
       <c r="B50" s="41" t="s">
-        <v>615</v>
+        <v>632</v>
       </c>
       <c r="C50" s="42" t="s">
-        <v>616</v>
+        <v>633</v>
       </c>
       <c r="D50" s="43">
         <v>9.9</v>
@@ -22950,10 +24786,10 @@
     <row r="51" spans="1:8">
       <c r="A51" s="40"/>
       <c r="B51" s="41" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="C51" s="42" t="s">
-        <v>617</v>
+        <v>634</v>
       </c>
       <c r="D51" s="43">
         <v>12.8</v>
@@ -22971,10 +24807,10 @@
         <v>46000</v>
       </c>
       <c r="B52" s="37" t="s">
-        <v>618</v>
+        <v>635</v>
       </c>
       <c r="C52" s="38" t="s">
-        <v>619</v>
+        <v>636</v>
       </c>
       <c r="D52" s="39">
         <v>24</v>
@@ -22993,10 +24829,10 @@
     <row r="53" spans="1:8">
       <c r="A53" s="36"/>
       <c r="B53" s="37" t="s">
-        <v>620</v>
+        <v>637</v>
       </c>
       <c r="C53" s="38" t="s">
-        <v>621</v>
+        <v>638</v>
       </c>
       <c r="D53" s="39">
         <v>12.2</v>
@@ -23012,10 +24848,10 @@
     <row r="54" spans="1:8">
       <c r="A54" s="36"/>
       <c r="B54" s="37" t="s">
-        <v>587</v>
+        <v>604</v>
       </c>
       <c r="C54" s="38" t="s">
-        <v>622</v>
+        <v>639</v>
       </c>
       <c r="D54" s="39">
         <v>13.4</v>
@@ -23033,10 +24869,10 @@
         <v>46001</v>
       </c>
       <c r="B55" s="41" t="s">
-        <v>602</v>
+        <v>619</v>
       </c>
       <c r="C55" s="42" t="s">
-        <v>623</v>
+        <v>640</v>
       </c>
       <c r="D55" s="43">
         <v>15.2</v>
@@ -23057,10 +24893,10 @@
         <v>46002</v>
       </c>
       <c r="B56" s="37" t="s">
-        <v>612</v>
+        <v>629</v>
       </c>
       <c r="C56" s="38" t="s">
-        <v>624</v>
+        <v>641</v>
       </c>
       <c r="D56" s="39">
         <v>12</v>
@@ -23078,10 +24914,10 @@
         <v>46010</v>
       </c>
       <c r="B57" s="49" t="s">
-        <v>625</v>
+        <v>642</v>
       </c>
       <c r="C57" s="50" t="s">
-        <v>626</v>
+        <v>643</v>
       </c>
       <c r="D57" s="51">
         <v>3.4</v>
@@ -23102,10 +24938,10 @@
         <v>46016</v>
       </c>
       <c r="B58" s="37" t="s">
-        <v>627</v>
+        <v>644</v>
       </c>
       <c r="C58" s="38" t="s">
-        <v>628</v>
+        <v>645</v>
       </c>
       <c r="D58" s="39">
         <v>14</v>
@@ -23126,10 +24962,10 @@
         <v>46016</v>
       </c>
       <c r="B59" s="37" t="s">
-        <v>541</v>
+        <v>558</v>
       </c>
       <c r="C59" s="38" t="s">
-        <v>629</v>
+        <v>646</v>
       </c>
       <c r="D59" s="39">
         <v>22</v>
@@ -23207,31 +25043,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>630</v>
+        <v>647</v>
       </c>
       <c r="C1" s="11" t="s">
-        <v>631</v>
+        <v>648</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>632</v>
+        <v>649</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>633</v>
+        <v>650</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>634</v>
+        <v>651</v>
       </c>
       <c r="G1" s="21" t="s">
-        <v>635</v>
+        <v>652</v>
       </c>
       <c r="H1" s="21" t="s">
-        <v>636</v>
+        <v>653</v>
       </c>
       <c r="I1" s="21" t="s">
-        <v>637</v>
+        <v>654</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>638</v>
+        <v>655</v>
       </c>
     </row>
     <row r="2" ht="126.7" customHeight="1" spans="1:10">
@@ -23239,16 +25075,16 @@
         <v>45967</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>639</v>
+        <v>656</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>640</v>
+        <v>657</v>
       </c>
       <c r="D2" s="15">
         <v>3</v>
       </c>
       <c r="E2" s="22" t="s">
-        <v>641</v>
+        <v>658</v>
       </c>
       <c r="F2" s="22"/>
       <c r="G2" s="23">
@@ -23263,7 +25099,7 @@
         <v>846000</v>
       </c>
       <c r="J2" s="22" t="s">
-        <v>642</v>
+        <v>659</v>
       </c>
     </row>
     <row r="3" ht="43" customHeight="1" spans="1:10">
@@ -23436,21 +25272,21 @@
   <sheetData>
     <row r="1" spans="2:3">
       <c r="B1" s="1" t="s">
-        <v>643</v>
+        <v>660</v>
       </c>
       <c r="C1" s="1"/>
     </row>
     <row r="2" spans="2:3">
       <c r="B2" s="1" t="s">
-        <v>644</v>
+        <v>661</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>645</v>
+        <v>662</v>
       </c>
     </row>
     <row r="3" spans="2:3">
       <c r="B3" s="2" t="s">
-        <v>646</v>
+        <v>663</v>
       </c>
       <c r="C3" s="2">
         <v>6699</v>
@@ -23458,7 +25294,7 @@
     </row>
     <row r="4" spans="2:3">
       <c r="B4" s="2" t="s">
-        <v>647</v>
+        <v>664</v>
       </c>
       <c r="C4" s="2">
         <v>2323</v>
@@ -23466,7 +25302,7 @@
     </row>
     <row r="5" spans="2:3">
       <c r="B5" s="2" t="s">
-        <v>648</v>
+        <v>665</v>
       </c>
       <c r="C5" s="2">
         <v>8899</v>
@@ -23474,7 +25310,7 @@
     </row>
     <row r="6" spans="2:3">
       <c r="B6" s="2" t="s">
-        <v>649</v>
+        <v>666</v>
       </c>
       <c r="C6" s="2">
         <v>5656</v>
@@ -23482,7 +25318,7 @@
     </row>
     <row r="7" spans="2:3">
       <c r="B7" s="2" t="s">
-        <v>650</v>
+        <v>667</v>
       </c>
       <c r="C7" s="2">
         <v>7744</v>
@@ -23490,7 +25326,7 @@
     </row>
     <row r="8" spans="2:3">
       <c r="B8" s="2" t="s">
-        <v>651</v>
+        <v>668</v>
       </c>
       <c r="C8" s="2">
         <v>4545</v>
@@ -23498,7 +25334,7 @@
     </row>
     <row r="9" spans="2:3">
       <c r="B9" s="2" t="s">
-        <v>652</v>
+        <v>669</v>
       </c>
       <c r="C9" s="2">
         <v>2525</v>
@@ -23506,7 +25342,7 @@
     </row>
     <row r="10" spans="2:3">
       <c r="B10" s="2" t="s">
-        <v>653</v>
+        <v>670</v>
       </c>
       <c r="C10" s="2">
         <v>3636</v>

</xml_diff>